<commit_message>
Updated eda_3 20260619 - dominance-sign_concordance matrix, classification, interpretation
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A2FA133-CF7E-5748-AF6E-4D96DF441DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98AC418A-C63F-3546-ACAF-C8A95D46A0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="133">
   <si>
     <t>Date</t>
   </si>
@@ -573,6 +573,129 @@
 4. Fig 14b flags an important limitation of the typology with large number of "Other change" MSOAs mainly distributed in outer North and East London. The typology is most analytically powerful for the inner-London areas, where cascade dynamics are strongest, and outer ring areas, where cross-decile flows are lower-volume and more volatile. </t>
     </r>
   </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If we have tested the rough symmetry between cascade and counter-cascade, then why the counter-cascade slightly dominates in London? -- This question is wrong, symmetry is about the response to the baseline reclassification.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2. Would the dominance of counter-led break the gentrification story in London?
+3. What's the relationship between the counter-led and the negative net_counter (divergent in sign concordance)?</t>
+    </r>
+  </si>
+  <si>
+    <t>§15b in eda_3;
+Net_cascade_counter matrix diagram.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Recall from Marcuse (1985), gentrification is a selective, localised process, where displacement is a neighbourhood-scale phenomenon operating within a broader urban system.
+2. From the study so far, we can understand the phenomenon as </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>a subset of neighbourhoods experience cascade-direction pressure, while the rest of the city absorbs the displaced population through the counter cascade direction</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+3. Combined with EDA_2, we have the spatial logic of a cascading system with net exporters and net absorbers. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Inner-city restructuring generates outward displacement, and the suburbs absorb it</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. The city-wide average tilts counter-cascade-led, because the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>displacement has to go somewhere, and "somewhere" is the numerical majority of London MSOAs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+4. There are noticeable excess of upward movers in 2011 (6%) and 2021 (13%). At every single decile, the share of outflows going to wealthier destinations exceeds the share of inflows from wealthier origins.
+5. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Gap of counter-dominance widened: A decade of inner-London gentrification had by 2021 already "completed" in many areas. Active cascade zones in 2011 were into settled, post-transition neighbourhoods.
+6. Counter-positive divergent is the strongest signal of displacement.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+** Given the "escalator effects" in London, how could displaced people move up to wealthier deciles? What's the underlying mechanism of that? Maybe this is out of scope of this study.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -581,7 +704,7 @@
   <numFmts count="1">
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -607,6 +730,13 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -1008,7 +1138,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" bestFit="1" customWidth="1"/>
@@ -1738,6 +1868,73 @@
       </c>
       <c r="H35" s="3" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="372" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
+        <v>46194</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
+        <v>46195</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
+        <v>46196</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
+        <v>46200</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
+        <v>46201</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
+        <v>46203</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
+        <v>46204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated eda_3 20260619 - dominance-sign_concordance matrix - new framework
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98AC418A-C63F-3546-ACAF-C8A95D46A0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01479303-0067-1443-BBED-67F98B350DF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="135">
   <si>
     <t>Date</t>
   </si>
@@ -572,37 +572,6 @@
       <t xml:space="preserve">.
 4. Fig 14b flags an important limitation of the typology with large number of "Other change" MSOAs mainly distributed in outer North and East London. The typology is most analytically powerful for the inner-London areas, where cascade dynamics are strongest, and outer ring areas, where cross-decile flows are lower-volume and more volatile. </t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t>1.</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> If we have tested the rough symmetry between cascade and counter-cascade, then why the counter-cascade slightly dominates in London? -- This question is wrong, symmetry is about the response to the baseline reclassification.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-2. Would the dominance of counter-led break the gentrification story in London?
-3. What's the relationship between the counter-led and the negative net_counter (divergent in sign concordance)?</t>
-    </r>
-  </si>
-  <si>
-    <t>§15b in eda_3;
-Net_cascade_counter matrix diagram.</t>
   </si>
   <si>
     <r>
@@ -695,6 +664,45 @@
       <t xml:space="preserve">
 ** Given the "escalator effects" in London, how could displaced people move up to wealthier deciles? What's the underlying mechanism of that? Maybe this is out of scope of this study.</t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> If we have tested the rough symmetry between cascade and counter-cascade, then why the counter-cascade slightly dominates in London? -- This question is wrong, symmetry is about the response to the baseline reclassification.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2. Would the dominance of counter-led break the gentrification story in London?
+3. What's the relationship between the counter-led and the negative net_counter (divergent in sign concordance)?
+4. How to understand the classification of MSOAs with both cascade_dominance and sign concordance?</t>
+    </r>
+  </si>
+  <si>
+    <t>1. How to understand the classification of MSOAs with both cascade_dominance and sign concordance?
+2. What do these classification distributed spatially?</t>
+  </si>
+  <si>
+    <t>Meeting with Adam for the next step direction.</t>
+  </si>
+  <si>
+    <t>§15c and §15d in eda_3;
+Net_cascade_counter matrix diagram.</t>
   </si>
 </sst>
 </file>
@@ -1878,13 +1886,19 @@
         <v>124</v>
       </c>
       <c r="D36" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E36" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="3" t="s">
         <v>132</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Start reprocess with London-touching flows; Finished §1&2
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C503937-2F37-2A43-A577-E5163410FE33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA92D4A-6B12-E142-82FE-1DD9E33AF7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="141">
   <si>
     <t>Date</t>
   </si>
@@ -537,9 +537,6 @@
   <si>
     <t>§14b in eda_3;
 §15b in eda_3.</t>
-  </si>
-  <si>
-    <t>Double check my design of cascade and counter-cascade. Do they fundamentally make sense? Would there be any problem in such design? If no, why counter-cascade dominated more, and we still have the tendency of more severe gentrification?</t>
   </si>
   <si>
     <t>EDA 3:
@@ -705,10 +702,102 @@
     <t xml:space="preserve">Meeting with Adam for the next step direction.
 Key findings need to be discussed at this stage:
 1. Counter-cascade flows (residents moving to less deprived areas) outweigh cascade flows (the gentrification-displacement direction) at every level of London's deprivation hierarchy in both 2011 and 2021, and the gap widened over the decade(EDA 2 §12b). ---EDA 2, §9, Fig 07; volume break down at EDA 3 §15c Panel (a)
-2. A four-type flow regime typology built from two independent dimensions (directional balance and cross-decile intensity, EDA 3 §12 Fig 12) significantly discriminates neighbourhood deprivation trajectories (Kruskal-Wallis p &lt; 0.001, EDA3 §18 Fig 17) and shows 58% structural persistence across the decade (EDA 3 §14b Fig 14b). 
-3. Cascade-led MSOAs nearly halved (130 → 72) between censuses, with the losses concentrated in inner south and west London's gentrification belt， suggesting many active displacement zones had "completed" their transition by 2021. --- EDA 3 §14
+2. A four-type flow regime typology built from two independent dimensions (directional balance and cross-decile intensity, EDA 3 §13 Fig 12) significantly discriminates neighbourhood deprivation trajectories (Kruskal-Wallis p &lt; 0.001, EDA3 §18 Fig 17) and shows 58% structural persistence across the decade (EDA 3 §15c Fig 14b). 
+3. Cascade-led MSOAs nearly halved (130 → 72) between censuses, with the losses concentrated in inner south and west London's gentrification belt， suggesting many active displacement zones had "completed" their transition by 2021. --- EDA 3 §14, §15c
 4. The IMD validation reveals that neighbourhoods losing their upwardly-mobile residents (counter-led) experience the strongest relative deprivation decline (Fig 17), while total migration churn (rho = 0.25) is a stronger predictor of neighbourhood change than directional dominance. Rrestructuring intensity matters more than direction. --- EDA3 Fig 16 and partial table in §17
 5. The ~10% of MSOAs with divergent sign concordance (EDA 1 §6c), particularly the counter-positive subtype (EDA 2 §11 Fig 09a/b) concentrated in inner-London boroughs like Newham and Hackney, represent the strongest displacement signal: areas haemorrhaging residents in both hierarchical directions simultaneously (EDA 3 §15c). </t>
+  </si>
+  <si>
+    <t>Adding outside London as a +1 MSOA;
+Compare with Duncan and/or Hong's work.
+(https://citygeographics.org/2022/12/15/tracking-gentrification-in-london-and-manchester-using-the-2021-census-occupational-class-data/)</t>
+  </si>
+  <si>
+    <t>1. If we introduce outside London in the migration analysis, would the counter overweigh cascade still been kept? Or we expect the cascade overweighs the counter?
+2. How would the difference between the comparison of attribute-detection and flow-detection? Why would the underlying reason be?
+3. Duncan's work doesn't have open resources, would it be better to use Yee's work?</t>
+  </si>
+  <si>
+    <t>Communication;
+Data preprocess;
+EDA</t>
+  </si>
+  <si>
+    <t>All questions raised before and key findings in yesterday's log;
+Would London-only internal analysis makes it a closed system for London? -- need national-frame extension.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Double check my design of cascade and counter-cascade. Do they fundamentally make sense? Would there be any problem in such design?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> If no, why counter-cascade dominated more, and we still have the tendency of more severe gentrification?</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">yee_lsoa_labels_from_repo.csv (all London LSOAs with classification labels, cloned from Yee's GitHub);
+ks101ew_lsoa_2011_allengland.csv
+data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb
+</t>
+  </si>
+  <si>
+    <r>
+      <t>Outside London is a big proportion missed so far, need to be analysed in the next step. -- High priority.
+Compare with attribute-based detections (Duncan Smith's work- professional change 2011-2021), there are some flagged areas in attribute-based dection, but shown as "Lateral" in current typology.
+1. London-relative analysis captures intra-urban restructuring. The national-frame analysis checks whether accounting for London's exchange with the rest of England changes the structural pattern. The two analyses are complementray. (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>London-relative result first, then national-frame extension to show if cascade/counter balance shifts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+2. London is more deprived than England on average. Comparing London and national wide, the internal deprivation hierarchy is preserved, but only the absolute position changes.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Most flows from outside London into London would register as `Inflow_Wealthier` (cascade direction), and most flows from London to outside will register as `Outflow_Wealthier`</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -718,7 +807,7 @@
   <numFmts count="1">
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -755,6 +844,11 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1875,13 +1969,13 @@
         <v>126</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G35" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="H35" s="3" t="s">
         <v>127</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="409" customHeight="1" x14ac:dyDescent="0.2">
@@ -1892,24 +1986,42 @@
         <v>124</v>
       </c>
       <c r="D36" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G36" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="H36" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="F36" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="1:8" ht="306" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>46195</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updateed reprocess of London-touching flows - national frame; Need to add more details from Churn analysis to start
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA92D4A-6B12-E142-82FE-1DD9E33AF7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18961424-6C94-8A40-BB1A-DEBD6EE6F4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="148">
   <si>
     <t>Date</t>
   </si>
@@ -797,6 +797,49 @@
         <scheme val="minor"/>
       </rPr>
       <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Data preprocess;
+EDA</t>
+  </si>
+  <si>
+    <t>data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb;
+</t>
+  </si>
+  <si>
+    <t>Does the national frame change narratives in London-only analysis?
+Where are those changes?
+How to understand those changes?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">msoa_cascade_national_frame_20260623.csv
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Where are those upward-mobility surplus MSOAs? DA_20260623, §5
+2. </t>
+  </si>
+  <si>
+    <r>
+      <t>1. National frame analysis confirmed "escalator effects" in London. London is a net exporter in both periods, and became more sharply in 2021. BUT, if comparing with attribute-based analysis, should consider both age and profession.
+2. In 2021, London's migration exchange is with the more affluent parts of England, rather than with the national average. Outflow destinations being slightly wealthier than inflow origins is consistent with the escalator model.
+3. Aggregated decile of all outside London MSOAs, in 2011 and 2021 it was D6. London exchanges with slightly wealthier-than-average England, not the "average England". 
+4. For 2021 OD data, during COVID, disproportionately sent residents to wealthier areas outside London.
+5.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> London's boundary is not a neutral container for the cascade/counter balance, and the direction of its effect changed between census periods. London-only analysis understates the counter-cascade shift in 2021. The core narrative (counter-cascade dominance intensifying between censuses, cascade as a localised perturbantion) holds even more firmly once accounting for boundary effects.</t>
     </r>
   </si>
 </sst>
@@ -2008,6 +2051,9 @@
       <c r="B37" s="3" t="s">
         <v>136</v>
       </c>
+      <c r="C37" s="3" t="s">
+        <v>142</v>
+      </c>
       <c r="D37" s="3" t="s">
         <v>137</v>
       </c>
@@ -2024,9 +2070,27 @@
         <v>134</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" ht="323" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>46196</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Finished data preprocess of national frame (adding external flows)
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18961424-6C94-8A40-BB1A-DEBD6EE6F4E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D318070-0064-6F47-86F5-86C20ECC246F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="150">
   <si>
     <t>Date</t>
   </si>
@@ -820,10 +820,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">1. Where are those upward-mobility surplus MSOAs? DA_20260623, §5
-2. </t>
-  </si>
-  <si>
     <r>
       <t>1. National frame analysis confirmed "escalator effects" in London. London is a net exporter in both periods, and became more sharply in 2021. BUT, if comparing with attribute-based analysis, should consider both age and profession.
 2. In 2021, London's migration exchange is with the more affluent parts of England, rather than with the national average. Outflow destinations being slightly wealthier than inflow origins is consistent with the escalator model.
@@ -840,6 +836,80 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> London's boundary is not a neutral container for the cascade/counter balance, and the direction of its effect changed between census periods. London-only analysis understates the counter-cascade shift in 2021. The core narrative (counter-cascade dominance intensifying between censuses, cascade as a localised perturbantion) holds even more firmly once accounting for boundary effects.</t>
+    </r>
+  </si>
+  <si>
+    <t>Where are those upward-mobility surplus MSOAs? DA_20260623, §5</t>
+  </si>
+  <si>
+    <t>Keep working on the national-frame analysis and compare with London-only analysis.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Both churns increase in national-frame because of the external flows added to the system, but there is asymmetry in the increase for different flows.
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The national-frame extension reveals that London's boundary effects are not temporally neutral.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In 2011, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>external flows</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> were roughly balanced between cascade and counter directions, leaving the London-only story essentially intact. By 2021, pandemic-era outmigration created a strong counter asymmetry in external flows, meaning the London-only analysis understates the counter-cascade intensification. (similar to finding 5 yesterday)
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Once classifying deciles natioanlly, London is more deprived.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Then within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4.
+4. When classifying flows within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4, so the same physical move might not corss a national decile boundary at all, or might cross it differently.</t>
     </r>
   </si>
 </sst>
@@ -2087,15 +2157,30 @@
         <v>145</v>
       </c>
       <c r="F38" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="G38" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="G38" s="3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H38" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="306" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>46197</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added eda_4 compare national-frame and London-only analysis
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D318070-0064-6F47-86F5-86C20ECC246F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BAAC652-5933-3841-810E-3A8EFB4C6554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="152">
   <si>
     <t>Date</t>
   </si>
@@ -911,6 +911,14 @@
       <t xml:space="preserve"> Then within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4.
 4. When classifying flows within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4, so the same physical move might not corss a national decile boundary at all, or might cross it differently.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_4_compare_natioanl_frame_and_london_only _20260624.ipynb
+</t>
+  </si>
+  <si>
+    <t>data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb;
+eda_4_compare_natioanl_frame_and_london_only _20260624.ipynb.</t>
   </si>
 </sst>
 </file>
@@ -2174,10 +2182,13 @@
         <v>141</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>144</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>150</v>
       </c>
       <c r="F39" s="3" t="s">
         <v>149</v>

</xml_diff>

<commit_message>
Updated eda4 - completed analysis and initial interpretation of part 1
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BAAC652-5933-3841-810E-3A8EFB4C6554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{736357E9-6921-7F42-8CF5-F638A86F9F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="153">
   <si>
     <t>Date</t>
   </si>
@@ -919,6 +919,10 @@
   <si>
     <t>data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb;
 eda_4_compare_natioanl_frame_and_london_only _20260624.ipynb.</t>
+  </si>
+  <si>
+    <t>1. Sign concordance changes in each cateogories from London-only to National-frame. Where are changes in spatial distribution?
+2. How to defend the design of aggregated outside London MSOAs' decile? We lost details that can be important. E.g. flows defined as OW can be actually OI, to an outside MSOA below D6?</t>
   </si>
 </sst>
 </file>
@@ -2193,6 +2197,9 @@
       <c r="F39" s="3" t="s">
         <v>149</v>
       </c>
+      <c r="G39" s="3" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="1">

</xml_diff>

<commit_message>
Added refined EDA 4 - split reclassification effects and external flow effects
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{736357E9-6921-7F42-8CF5-F638A86F9F15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FE4604-A5F5-6E4E-8028-7D0B503B74A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="154">
   <si>
     <t>Date</t>
   </si>
@@ -845,74 +845,6 @@
     <t>Keep working on the national-frame analysis and compare with London-only analysis.</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">1. Both churns increase in national-frame because of the external flows added to the system, but there is asymmetry in the increase for different flows.
-2. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>The national-frame extension reveals that London's boundary effects are not temporally neutral.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> In 2011, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>external flows</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> were roughly balanced between cascade and counter directions, leaving the London-only story essentially intact. By 2021, pandemic-era outmigration created a strong counter asymmetry in external flows, meaning the London-only analysis understates the counter-cascade intensification. (similar to finding 5 yesterday)
-3. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Once classifying deciles natioanlly, London is more deprived.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Then within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4.
-4. When classifying flows within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4, so the same physical move might not corss a national decile boundary at all, or might cross it differently.</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">eda_4_compare_natioanl_frame_and_london_only _20260624.ipynb
 </t>
   </si>
@@ -921,8 +853,248 @@
 eda_4_compare_natioanl_frame_and_london_only _20260624.ipynb.</t>
   </si>
   <si>
-    <t>1. Sign concordance changes in each cateogories from London-only to National-frame. Where are changes in spatial distribution?
-2. How to defend the design of aggregated outside London MSOAs' decile? We lost details that can be important. E.g. flows defined as OW can be actually OI, to an outside MSOA below D6?</t>
+    <r>
+      <t xml:space="preserve">1. Sign concordance changes in each cateogories from London-only to National-frame. Where are changes in spatial distribution? -- </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>They are disclosure-suppressed MSOAs with no migration data in 2021, and they exist in both frames identically. (Solved)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2. How to defend the design of aggregated outside London MSOAs' decile? We lost details that can be important. E.g. flows defined as OW can be actually OI, to an outside MSOA below D6?
+3. The key question after counter analysis: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">why do most flows move toward wealthier neighbourhoods? </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Three hypothesis are: a) residential aspiration - people are generally prefer less deprived neighbourhoods; b) housing ladder effect - households move as income rises (inner deprived area - suburb middle area - affluent suburb); c) London suburbanisation after COVID
+4. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>If counter-cascade flows are the norm, what makes a neighbourhood cascade-dominant?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+5. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Which neighbourhoods systematically attract migrants from lower-deprivation origins despite the overall tendency for households to move up the deprivation hierarchy?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+6. Choice of using IMD to represent deprivation? Should have denfense on this in the dissertation. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. There is asymmetry in the increase for different flows.
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The national-frame extension reveals that London's boundary effects are not temporally neutral.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> In 2011, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>external flows</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> were roughly balanced between cascade/counter directions, leaving the London-only story essentially intact. By 2021, pandemic-era outmigration created a strong counter asymmetry in external flows, meaning the London-only analysis understates the counter-cascade intensification.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Once classifying deciles natioanlly, London is more deprived.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Then within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4.
+4. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">National D6 aggregation for all outside London MSOAs is a limitation, but validated by the data repreprocess file. For any individual MSOA, the actual composition of its external exchange partners could deviate substantially from D6. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> It's a reasonable simplification that preserves the structure of London-facing migration flows
+5. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>London's internal hierarchy is more differentiated than the national one.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> When classifying flows within a London-only frame, a move from London D5 to London D6 crosses one decile boundary. But nationally, both of those areas might sits in national D3-D4, so the same physical move might not corss a national decile boundary at all, or might cross it differently.
+6. (Interpretation cell in part 1e in EDA_4.) 
+7. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The choice of decile reference frame barely alters the balance between cascade and counter-cascade</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Whether the observed counter shift comes primarily from London-to-outside, or outside-to-London, or within London?
+Given the counter dominance was intensified both temporally and by addition of external flows, we need to:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1. Establish overall migration direction.
+2. Compare London-only and National-framw.
+3. Identify the most cascade-dominant MSOAs and the most counter-dominant MSOAs in both years.
+4. Examine whether those deviations correspond with other restructuring indicators (attribute-based) - What kinds of neighbourhoods systematically deviate from the metropolitan baseline?
+5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Explain reasons of those deviations.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -932,7 +1104,7 @@
   <numFmts count="1">
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -974,6 +1146,18 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2178,7 +2362,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="306" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>46197</v>
       </c>
@@ -2186,19 +2370,22 @@
         <v>141</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>144</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Paused refined EDA 4 - need a refined preprocess for 2021 flows' geography with 2011 codes
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FE4604-A5F5-6E4E-8028-7D0B503B74A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CF5D9D-253A-8F46-A6BF-6732681A7FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="159">
   <si>
     <t>Date</t>
   </si>
@@ -1095,6 +1095,26 @@
       </rPr>
       <t>. Explain reasons of those deviations.</t>
     </r>
+  </si>
+  <si>
+    <t>1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
+2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Need a refined data preprocess file for 2021 flows converted back to 2011 geography.
+</t>
+  </si>
+  <si>
+    <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
+eda_4(2nd-draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. 
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. How to deal with those missing 20 MSOAs in 2021 records? The key principle is to use 2011 MSOAs as the analysis unit. 2021 flows should be converted back to 2011 geogeaphy.
+2. </t>
   </si>
 </sst>
 </file>
@@ -2388,9 +2408,30 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added a data preprocess check for 20 missing msoas in 2021 od data
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78CF5D9D-253A-8F46-A6BF-6732681A7FE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046E6D94-96E7-AC49-9264-6B8F2EF5E37C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="160">
   <si>
     <t>Date</t>
   </si>
@@ -1097,10 +1097,6 @@
     </r>
   </si>
   <si>
-    <t>1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
-2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file.</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Need a refined data preprocess file for 2021 flows converted back to 2011 geography.
 </t>
   </si>
@@ -1115,6 +1111,37 @@
   <si>
     <t xml:space="preserve">1. How to deal with those missing 20 MSOAs in 2021 records? The key principle is to use 2011 MSOAs as the analysis unit. 2021 flows should be converted back to 2011 geogeaphy.
 2. </t>
+  </si>
+  <si>
+    <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
+eda_4(2nd-draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
+datat_preprocess_20_missing_msoas_only_in_2021_20260625.ipynb</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
+2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2408,7 +2435,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="204" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>
@@ -2416,22 +2443,22 @@
         <v>141</v>
       </c>
       <c r="C40" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G40" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="D40" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="F40" s="3" t="s">
+      <c r="H40" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Finished data repreprocess - geo harmonise for 2021 msoa for 20260615 preprocess file
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{046E6D94-96E7-AC49-9264-6B8F2EF5E37C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92FD1A3-FCDE-F449-873D-3CDF2756BD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1113,35 +1113,39 @@
 2. </t>
   </si>
   <si>
+    <r>
+      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
+2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+  </si>
+  <si>
     <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
 eda_4(2nd-draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
-datat_preprocess_20_missing_msoas_only_in_2021_20260625.ipynb</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
-2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
+datat_preprocess_20_missing_msoas_only_in_2021_20260625.ipynb;
+geo_harmonisation_remap_audit.csv (output);
+data_preprocess_geo_harmonise_2021_msoa_missing_solved_from_20260615version_20260625.ipynb;
+exclusion_summary_20260625.csv (output);
+msoa_cascade_features_20260625.csv (output)</t>
   </si>
 </sst>
 </file>
@@ -2435,7 +2439,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="238" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>
@@ -2449,10 +2453,10 @@
         <v>157</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>159</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
Finished rerun EDA_1 with findings in changes recorded in the research logbook
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92FD1A3-FCDE-F449-873D-3CDF2756BD4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65143FC9-C1DB-634C-A48C-A430DFBE84B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1113,32 +1113,6 @@
 2. </t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
-2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-  </si>
-  <si>
     <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
 eda_4(2nd-draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
 datat_preprocess_20_missing_msoas_only_in_2021_20260625.ipynb;
@@ -1146,6 +1120,53 @@
 data_preprocess_geo_harmonise_2021_msoa_missing_solved_from_20260615version_20260625.ipynb;
 exclusion_summary_20260625.csv (output);
 msoa_cascade_features_20260625.csv (output)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
+2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>After redo data preprocess, EDA_1 has significant changes in cross-decile share plot (fig4), but cascade dominance look almost identical</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. For sign concordance, more Divergent (101) MSOAs and only 3 Zero (21 before).</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2439,7 +2460,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="238" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="272" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>
@@ -2453,10 +2474,10 @@
         <v>157</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>158</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
Rerun EDA 2 - need more refined interpretation on figs. Most findings are unchanges, need explorations on cross-decile share.
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65143FC9-C1DB-634C-A48C-A430DFBE84B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0E1442-47E6-D944-83DD-F7D6A09FB7F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1097,20 +1097,12 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1. Need a refined data preprocess file for 2021 flows converted back to 2011 geography.
-</t>
-  </si>
-  <si>
     <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
 eda_4(2nd-draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb</t>
   </si>
   <si>
     <t xml:space="preserve">1. 
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. How to deal with those missing 20 MSOAs in 2021 records? The key principle is to use 2011 MSOAs as the analysis unit. 2021 flows should be converted back to 2011 geogeaphy.
-2. </t>
   </si>
   <si>
     <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
@@ -1122,6 +1114,10 @@
 msoa_cascade_features_20260625.csv (output)</t>
   </si>
   <si>
+    <t>1. How to deal with those missing 20 MSOAs in 2021 records? The key principle is to use 2011 MSOAs as the analysis unit. 2021 flows should be converted back to 2011 geogeaphy.
+2. After new data preprocessed file, what are the changes in the rerun EDA 1-3?</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
 2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
@@ -1155,7 +1151,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>After redo data preprocess, EDA_1 has significant changes in cross-decile share plot (fig4), but cascade dominance look almost identical</t>
+      <t>After redo data preprocess, rerun EDA_1 has significant changes in cross-decile share plot (fig4), but cascade dominance look almost identical</t>
     </r>
     <r>
       <rPr>
@@ -1165,8 +1161,36 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>. For sign concordance, more Divergent (101) MSOAs and only 3 Zero (21 before).</t>
-    </r>
+      <t>. For sign concordance, more Divergent (101) MSOAs and only 3 Zero (21 before).
+4. London-only analysis sign concordant, aligning with London's deprivation gradient: [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EDA2§11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>]divergent MSOAs growth amount are the same in the sign concordance analysis, but more cascade-positive (net receivers).</t>
+    </r>
+  </si>
+  <si>
+    <t>0. Understand the rerun differences?
+1. Interpret changes in rerun EDAs. 
+    - EDA_2-section 8, fig 7 cds; fig 8; fig 9a; fig 10 black lines + divergent MSOAs in 2021; fig 11
+2. Interpretations can be merged and refined:
+- EDA_2 - §11 - divergent subtype interpretation</t>
   </si>
 </sst>
 </file>
@@ -2460,7 +2484,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="272" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="340" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>
@@ -2468,22 +2492,22 @@
         <v>141</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>157</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="G40" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="H40" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Rerun EDA 3 - need more refined interpretation on figs. Most findings are unchanges.
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F0E1442-47E6-D944-83DD-F7D6A09FB7F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C3A539-3A05-5841-B448-1450D89FCDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1101,8 +1101,109 @@
 eda_4(2nd-draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb</t>
   </si>
   <si>
-    <t xml:space="preserve">1. 
+    <t>1. How to deal with those missing 20 MSOAs in 2021 records? The key principle is to use 2011 MSOAs as the analysis unit. 2021 flows should be converted back to 2011 geogeaphy.
+2. After new data preprocessed file, what are the changes in the rerun EDA 1-3?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. There are significant changes in cross-decile share after rerun and correct geo harmonisation. It seems previous COVID-related reasons are not valid in 2021, as they shared the similar pattern with 2011. How to understand this now? COVID actually does not that a big deal?
 </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
+2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>After redo data preprocess, rerun EDA_1 has significant changes in cross-decile share plot (fig4), but cascade dominance look almost identical</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. For sign concordance, more Divergent (101) MSOAs and only 3 Zero (21 before).
+4. London-only analysis sign concordant, aligning with London's deprivation gradient: [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EDA2§11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">]divergent MSOAs growth amount are the same in the sign concordance analysis, but more cascade-positive (net receivers).
+5. London-only analysis new typology (dominance-sign_concordance) have more detailed </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>borough-level analysis on restructuring</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - rerun EDA_3 - §16.</t>
+    </r>
+  </si>
+  <si>
+    <t>0. Understand the rerun differences?
+1. Interpret changes in rerun EDAs. 
+    - EDA_2 - section 8; fig 7 cds; fig 8; fig 9a; fig 10 black lines + divergent MSOAs in 2021; fig 11
+    - EDA_3 - §13 stats; fig 12; fig 13; fig 13b; fig 14c (b); §15c final interpretation need split categories in `Concordant`; fig 16; 
+2. Interpretations can be merged and refined:
+- EDA_2 - §11 - divergent subtype interpretation</t>
   </si>
   <si>
     <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
@@ -1111,86 +1212,9 @@
 geo_harmonisation_remap_audit.csv (output);
 data_preprocess_geo_harmonise_2021_msoa_missing_solved_from_20260615version_20260625.ipynb;
 exclusion_summary_20260625.csv (output);
-msoa_cascade_features_20260625.csv (output)</t>
-  </si>
-  <si>
-    <t>1. How to deal with those missing 20 MSOAs in 2021 records? The key principle is to use 2011 MSOAs as the analysis unit. 2021 flows should be converted back to 2011 geogeaphy.
-2. After new data preprocessed file, what are the changes in the rerun EDA 1-3?</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
-2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 
-3. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>After redo data preprocess, rerun EDA_1 has significant changes in cross-decile share plot (fig4), but cascade dominance look almost identical</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. For sign concordance, more Divergent (101) MSOAs and only 3 Zero (21 before).
-4. London-only analysis sign concordant, aligning with London's deprivation gradient: [</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>EDA2§11</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>]divergent MSOAs growth amount are the same in the sign concordance analysis, but more cascade-positive (net receivers).</t>
-    </r>
-  </si>
-  <si>
-    <t>0. Understand the rerun differences?
-1. Interpret changes in rerun EDAs. 
-    - EDA_2-section 8, fig 7 cds; fig 8; fig 9a; fig 10 black lines + divergent MSOAs in 2021; fig 11
-2. Interpretations can be merged and refined:
-- EDA_2 - §11 - divergent subtype interpretation</t>
+msoa_cascade_features_20260625.csv (output);
+msoa_typology_labels_20260625.csv (output);
+3 rerun EDA_1 to EDA_3</t>
   </si>
 </sst>
 </file>
@@ -2484,7 +2508,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="340" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="388" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>
@@ -2495,19 +2519,19 @@
         <v>154</v>
       </c>
       <c r="D40" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F40" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="G40" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="H40" s="3" t="s">
         <v>158</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added rerun data preprocess with national frame - have a bug in section 3 step 4.
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C3A539-3A05-5841-B448-1450D89FCDD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8B7BA4-1977-0E40-A059-8C79B97CA2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1214,7 +1214,8 @@
 exclusion_summary_20260625.csv (output);
 msoa_cascade_features_20260625.csv (output);
 msoa_typology_labels_20260625.csv (output);
-3 rerun EDA_1 to EDA_3</t>
+3 rerun EDA_1 to EDA_3;
+data_preprocess_rerun_national_frame_20260625.ipynb;</t>
   </si>
 </sst>
 </file>
@@ -1679,11 +1680,11 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.1640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="39.83203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="58.5" style="2" customWidth="1"/>
-    <col min="5" max="5" width="43.5" style="2" customWidth="1"/>
-    <col min="6" max="6" width="73.1640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="75.1640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="89.5" style="2" customWidth="1"/>
+    <col min="6" max="6" width="111.5" style="2" customWidth="1"/>
     <col min="7" max="7" width="59.83203125" style="2" customWidth="1"/>
     <col min="8" max="8" width="63" style="2" customWidth="1"/>
     <col min="9" max="16384" width="10.83203125" style="2"/>

</xml_diff>

<commit_message>
Added rerun EDA 4 with new harmonised df - paused at section 1c
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8B7BA4-1977-0E40-A059-8C79B97CA2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DCC9B4F-6D9F-8946-A754-0DE8C1FFDA13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1198,12 +1198,32 @@
     </r>
   </si>
   <si>
-    <t>0. Understand the rerun differences?
+    <r>
+      <t xml:space="preserve">0. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Understand the changes in cross-decile shares</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.
 1. Interpret changes in rerun EDAs. 
     - EDA_2 - section 8; fig 7 cds; fig 8; fig 9a; fig 10 black lines + divergent MSOAs in 2021; fig 11
     - EDA_3 - §13 stats; fig 12; fig 13; fig 13b; fig 14c (b); §15c final interpretation need split categories in `Concordant`; fig 16; 
 2. Interpretations can be merged and refined:
 - EDA_2 - §11 - divergent subtype interpretation</t>
+    </r>
   </si>
   <si>
     <t>eda_4(draft-refine)compare_natioanl_frame_and_london_only_20260625.ipynb;
@@ -1214,8 +1234,10 @@
 exclusion_summary_20260625.csv (output);
 msoa_cascade_features_20260625.csv (output);
 msoa_typology_labels_20260625.csv (output);
+msoa_cascade_national_frame_20260625.csv (output);
 3 rerun EDA_1 to EDA_3;
-data_preprocess_rerun_national_frame_20260625.ipynb;</t>
+data_preprocess_rerun_national_frame_20260625.ipynb;
+geo_harmonise.py (iterated);</t>
   </si>
 </sst>
 </file>
@@ -2509,7 +2531,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="388" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="272" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>

</xml_diff>

<commit_message>
Updated rerun EDA 4 with new harmonised df
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DCC9B4F-6D9F-8946-A754-0DE8C1FFDA13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F162A381-19D8-B840-9D99-3706290AB0EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="162">
   <si>
     <t>Date</t>
   </si>
@@ -1235,9 +1235,39 @@
 msoa_cascade_features_20260625.csv (output);
 msoa_typology_labels_20260625.csv (output);
 msoa_cascade_national_frame_20260625.csv (output);
-3 rerun EDA_1 to EDA_3;
+3 rerun EDA_1 to EDA_4;
 data_preprocess_rerun_national_frame_20260625.ipynb;
 geo_harmonise.py (iterated);</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_4_rerun_compare_natioanl_frame_and_london_only__20260625.ipynb;
+</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Over the census periods, there are more external flows in both direction from every deciles</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. D1 attracted more external inflows in 2011, but it became more outflow dominated by 2021.
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2557,9 +2587,18 @@
         <v>158</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>46199</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated rerun EDA 4 with new harmonised df - part 1 done.
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F162A381-19D8-B840-9D99-3706290AB0EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A3474D-7BBF-EC42-A1DA-0FB1BCECCD3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="900" windowWidth="28040" windowHeight="17180" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="15140" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="163">
   <si>
     <t>Date</t>
   </si>
@@ -1244,6 +1244,9 @@
 </t>
   </si>
   <si>
+    <t>What drives the 2011 to 2021 counter shift?</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">1. </t>
     </r>
@@ -1266,6 +1269,114 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">. D1 attracted more external inflows in 2011, but it became more outflow dominated by 2021.
+2. Compared with 2011, external counter boost bars dwarf in 2021, while relassification changes stay similar across years. (EDA4-1e)
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">It is the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>London to external migration drives the counter shift</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> from 2011 to 2021</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, which broke our expectation of cascade shift with external flow coming in the analysis. London internal reshuffling is a secondary factor. Both the cascade and counter component of external to London flow decreased, meaning the</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> total overall inflow to London from the rest of the country shrank. 
+Even internal city churn making up the largest baseline volume of people, temporal changes are relatively modest, compared with London-external temporal changes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">4. Fig 20b in EDA_4 helps justify the choice of London-only analysis as the main one, and the national-frame analysis as a complemenatry context. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>The core story is "How is London reshaping itself?" Then transitioning with "London is certainly not a vacuum". Then introducing external flows to show how the system boundaries are leaking - While internal churn remained high, the actual shift in the counter-trend was heavily impacted by an exodus of people leaving the city entirely</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
 </t>
     </r>
   </si>
@@ -1277,7 +1388,7 @@
   <numFmts count="1">
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1331,6 +1442,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2587,7 +2704,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" ht="272" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>46199</v>
       </c>
@@ -2597,8 +2714,11 @@
       <c r="C41" s="3" t="s">
         <v>160</v>
       </c>
+      <c r="D41" s="2" t="s">
+        <v>161</v>
+      </c>
       <c r="F41" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated rerun EDA 4 with new harmonised df - part 2 done.
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9A3474D-7BBF-EC42-A1DA-0FB1BCECCD3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54787E10-C42B-B348-9A2C-7632DF376DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15140" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="165">
   <si>
     <t>Date</t>
   </si>
@@ -1107,95 +1107,6 @@
   <si>
     <t xml:space="preserve">1. There are significant changes in cross-decile share after rerun and correct geo harmonisation. It seems previous COVID-related reasons are not valid in 2021, as they shared the similar pattern with 2011. How to understand this now? COVID actually does not that a big deal?
 </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
-2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. 
-3. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>After redo data preprocess, rerun EDA_1 has significant changes in cross-decile share plot (fig4), but cascade dominance look almost identical</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. For sign concordance, more Divergent (101) MSOAs and only 3 Zero (21 before).
-4. London-only analysis sign concordant, aligning with London's deprivation gradient: [</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>EDA2§11</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">]divergent MSOAs growth amount are the same in the sign concordance analysis, but more cascade-positive (net receivers).
-5. London-only analysis new typology (dominance-sign_concordance) have more detailed </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>borough-level analysis on restructuring</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> - rerun EDA_3 - §16.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -1247,6 +1158,124 @@
     <t>What drives the 2011 to 2021 counter shift?</t>
   </si>
   <si>
+    <t xml:space="preserve">1. Is the hypothesis true with external flows that "People moving into or out of the city were vastly more likely to be involved in moves toward wealthier deciles than in 2011?" What are the counts for London-only analysis?
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Need to check in sign concordance matrix with external flows, how many are concordant with positive, defined as upward-connected hubs. And compare with London-only analysis, to check today's blue finding 5.
+</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
+2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Camden 024 and Camden 025 were merged into one 2021 MSOA, they are analysed as a single best-fit combined zone across both census years to preserve a consistent spatial framework; this affects 2 of 983 units and leaves the deprivation-decile structure of all other areas unchanged</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. 
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>After redo data preprocess, rerun EDA_1 has significant changes in cross-decile share plot (fig4), but cascade dominance look almost identical</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. For sign concordance, more Divergent (101) MSOAs and only 3 Zero (21 before).
+4. London-only analysis sign concordant, aligning with London's deprivation gradient: [</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>EDA2§11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">]divergent MSOAs growth amount are the same in the sign concordance analysis, but more cascade-positive (net receivers).
+5. London-only analysis new typology (dominance-sign_concordance) have more detailed </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>borough-level analysis on restructuring</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - rerun EDA_3 - §16.
+6. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>~69.1% London MSOAs are below national D6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (data_preprocess_rerun_national_frame_20260625.ipynb).</t>
+    </r>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">1. </t>
     </r>
@@ -1366,7 +1395,84 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>.</t>
+      <t xml:space="preserve">.
+5. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Reclassification and relative more deprived MSOAs in London makes Churn and Cross-decile share drop</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. By 2021, London's interaction with the outside neighbourhoods became highly skewed toward "counter" (upward) mobility. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>People moving into or out of the city were vastly more likely to be involved in moves toward wealthier deciles than in 2011 (sign concordance checked, EDA_4 - 2d)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+6. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">External migration acts opposite (divergent) on cascade/counter dominance push between London's wealthier (toward cascade) and poorer (toward counter) neighbourhoods, with a clear structural split </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(fig 21). ~69.1% London MSOAs are below national D6. Because the vast majority of London's neighbourhoods are concentrated in the lower deciles, the counter push exerted by external flows on these specific areas completely overwhelms the extreme.
+7. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>External migration have opposite (divergent) effects on number of "Net receiver" and "Net exporter" over the periods.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Net receiver decreased 60%, Net exporter increased 118%. Withour external flows, reclassification affects very subtly.</t>
     </r>
     <r>
       <rPr>
@@ -2678,7 +2784,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="272" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" ht="306" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>
@@ -2692,19 +2798,19 @@
         <v>155</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>156</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="272" x14ac:dyDescent="0.2">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>46199</v>
       </c>
@@ -2712,12 +2818,18 @@
         <v>10</v>
       </c>
       <c r="C41" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="F41" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="G41" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="H41" s="3" t="s">
         <v>162</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Completed rerun EDA 4 with new harmonised df
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54787E10-C42B-B348-9A2C-7632DF376DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7287D641-899D-DF46-9197-97C3D0D4A35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="166">
   <si>
     <t>Date</t>
   </si>
@@ -1158,14 +1158,6 @@
     <t>What drives the 2011 to 2021 counter shift?</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Is the hypothesis true with external flows that "People moving into or out of the city were vastly more likely to be involved in moves toward wealthier deciles than in 2011?" What are the counts for London-only analysis?
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Need to check in sign concordance matrix with external flows, how many are concordant with positive, defined as upward-connected hubs. And compare with London-only analysis, to check today's blue finding 5.
-</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
 2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
@@ -1274,6 +1266,10 @@
       </rPr>
       <t xml:space="preserve"> (data_preprocess_rerun_national_frame_20260625.ipynb).</t>
     </r>
+  </si>
+  <si>
+    <t>1. Is the hypothesis true with external flows that "People moving into or out of the city were vastly more likely to be involved in moves toward wealthier deciles than in 2011?" What are the counts for London-only analysis? --- yes, confirmed with people volumes in the same result.
+2. (Typology) Reclassification and external flow effects on the increase or the decrease of cascade-led and counter-led? And there is a big drop of symmetric with external flows.</t>
   </si>
   <si>
     <r>
@@ -1423,7 +1419,7 @@
         <color rgb="FFFF0000"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>People moving into or out of the city were vastly more likely to be involved in moves toward wealthier deciles than in 2011 (sign concordance checked, EDA_4 - 2d)</t>
+      <t>People moving into or out of the city were vastly more likely to be involved in moves toward wealthier deciles than in 2011</t>
     </r>
     <r>
       <rPr>
@@ -1472,7 +1468,81 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> Net receiver decreased 60%, Net exporter increased 118%. Withour external flows, reclassification affects very subtly.</t>
+      <t xml:space="preserve"> Net receiver decreased 60%, Net exporter increased 118%. Withour external flows, reclassification affects very subtly.
+8. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>More cascade-led MSOAs in national-frame analysis than the London-only analysis for both census periods</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. But, the cacade dominance still shows as counter-dominated. We can say even the count of cascade-led increase, the counter-led norm is still undeniable in London.
+9. Through national lens, London's neighbourhoods have become highly polarized in migration flows.
+10. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Cascade inner-to-outer shift on map is not gentrification relocaing, it's a change in which process domiantes the metrics, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">it's mainly because the pandemic exodus(fig 25, table in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>part 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Map of extreme MSOAs in last section in EDA_4 (Done).</t>
     </r>
     <r>
       <rPr>
@@ -1483,8 +1553,33 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Part 4 and Fig 20b in EDA_4 proved using London-only analysis as the core analysis, and national frame as the complementary one</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">eda4_results_for_phase3_20260626.csv (output);
+All figs from EDA_4 (rerun_eda_figs_20260625)
 </t>
-    </r>
   </si>
 </sst>
 </file>
@@ -1959,7 +2054,7 @@
     <col min="3" max="3" width="37.1640625" style="2" customWidth="1"/>
     <col min="4" max="4" width="75.1640625" style="2" customWidth="1"/>
     <col min="5" max="5" width="89.5" style="2" customWidth="1"/>
-    <col min="6" max="6" width="111.5" style="2" customWidth="1"/>
+    <col min="6" max="6" width="151.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="59.83203125" style="2" customWidth="1"/>
     <col min="8" max="8" width="63" style="2" customWidth="1"/>
     <col min="9" max="16384" width="10.83203125" style="2"/>
@@ -2801,7 +2896,7 @@
         <v>158</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>156</v>
@@ -2823,14 +2918,17 @@
       <c r="D41" s="2" t="s">
         <v>160</v>
       </c>
+      <c r="E41" s="3" t="s">
+        <v>165</v>
+      </c>
       <c r="F41" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>164</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added 2011 and 2021 occupation data for comparison with occupational analysis
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7287D641-899D-DF46-9197-97C3D0D4A35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849F49BD-22D2-794C-A9EE-90BEA57476D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="170">
   <si>
     <t>Date</t>
   </si>
@@ -1155,9 +1155,6 @@
 </t>
   </si>
   <si>
-    <t>What drives the 2011 to 2021 counter shift?</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1. In both 2011 and 2021, the ladder reclassification makes the system shift toward cascade. But adding external flows have opposite effects in 2021 (harder counter push) and 2011 (more cascade nudge), and even large enough for 2021 to flip the net shift's sign.
 2. 20 MSOAs in 2021 with literally zero recorded migration, are exactly London 2011 codes absent from the raw 2021 file. 18 MSOAs were split in 2021, and 2 were merged. Split cases are easy to deal with, but we decided that </t>
@@ -1270,6 +1267,61 @@
   <si>
     <t>1. Is the hypothesis true with external flows that "People moving into or out of the city were vastly more likely to be involved in moves toward wealthier deciles than in 2011?" What are the counts for London-only analysis? --- yes, confirmed with people volumes in the same result.
 2. (Typology) Reclassification and external flow effects on the increase or the decrease of cascade-led and counter-led? And there is a big drop of symmetric with external flows.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Map of extreme MSOAs in last section in EDA_4 (Done).</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Part 4 and Fig 20b in EDA_4 proved using London-only analysis as the core analysis, and national frame as the complementary one</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">eda4_results_for_phase3_20260626.csv (output);
+All figs from EDA_4 (rerun_eda_figs_20260625)
+</t>
+  </si>
+  <si>
+    <t>What drives the 2011 to 2021 counter shift?
+Where are most cascade or counter dominated MSOAs? Any changes over the periods?</t>
   </si>
   <si>
     <r>
@@ -1496,28 +1548,46 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Cascade inner-to-outer shift on map is not gentrification relocaing, it's a change in which process domiantes the metrics, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">it's mainly because the pandemic exodus(fig 25, table in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
         <color rgb="FFFF0000"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
+      <t>Cascade inner-to-outer shift on map is not gentrification relocaing, it's a change in which process domiantes the metrics</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>it's mainly because the pandemic exodus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(fig 25, table in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
       <t>part 4</t>
     </r>
     <r>
@@ -1532,38 +1602,37 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">0. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Need to specify in the methodology chapter about the convention of Net counter, Cascade-Inflow-share, Pct_Inflow_Wealthier;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">
-1. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Map of extreme MSOAs in last section in EDA_4 (Done).</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
+1. Add borough names on the map for better readability
 2. </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Part 4 and Fig 20b in EDA_4 proved using London-only analysis as the core analysis, and national frame as the complementary one</t>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Confirm with Duncan about the SOC major groups he used</t>
     </r>
     <r>
       <rPr>
@@ -1577,9 +1646,102 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">eda4_results_for_phase3_20260626.csv (output);
-All figs from EDA_4 (rerun_eda_figs_20260625)
+    <t xml:space="preserve">2011_occupation_msoa.csv (data);
+2021_occupation_msoa.csv (data);
 </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. I have a feeling to use London-only analysis as the core analysis, and we had some evidence from yesterday's findings, but logically, how does it make sense?
+2. Double check all EDA 1-4 results so far before any comparison work.
+3. How to select and compare our work with attibute-based analysis work? Yee's work in for 2011, but Duncan's code and analysis work is not public, we just have his article report.
+ - Duncan's work is mainly about changes in share of residents in the top occupationaly class from 2011 to 2021.
+- Compare stats - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Cramér's V and Adjusted Rand Index</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> - measuring association or agreement between 2 categorical classifications. "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Do my flow typology and Yee's gentrification typology carve London into similar groups?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">0. Net Counter = Outflow_Wealthier - Inflow_Poorer, so positive Net_Counter means more people move to wealthier areas than people moving from poorer areas. Need to watch out the logic.
+1. For replication of Duncan's work, the ONS table page for the 2021 NS-SeC (TS062) explicitly warns it's not comparable with the 2011 Census because the classifications in the occupation variable have changed. So we need to replicate the usage of SOC major group (1 Managers/Directors, 2 Professional, 3 Associate Professional), rather than NS-SeC.
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>2021 cascade-dominance shift is not tracking attribute-gentrification, it's flow restructuring [exodus]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (from </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uncorrelation between affluent share change and IMD change in occupational analysis comparison</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, consistent with finding 10 yesterday).</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1589,7 +1751,7 @@
   <numFmts count="1">
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1648,6 +1810,12 @@
       <b/>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow (Body)"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF00B0F0"/>
       <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
@@ -2896,7 +3064,7 @@
         <v>158</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>156</v>
@@ -2915,25 +3083,37 @@
       <c r="C41" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>160</v>
+      <c r="D41" s="3" t="s">
+        <v>164</v>
       </c>
       <c r="E41" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="F41" s="3" t="s">
-        <v>163</v>
-      </c>
       <c r="G41" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="H41" s="3" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:8" ht="204" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>46200</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added 2011 LSOA-to-MSOA map output
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849F49BD-22D2-794C-A9EE-90BEA57476D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9F536B-7829-F843-B84E-22FAA23BE9AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1646,11 +1646,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">2011_occupation_msoa.csv (data);
-2021_occupation_msoa.csv (data);
-</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1. I have a feeling to use London-only analysis as the core analysis, and we had some evidence from yesterday's findings, but logically, how does it make sense?
 2. Double check all EDA 1-4 results so far before any comparison work.
@@ -1742,6 +1737,11 @@
       </rPr>
       <t>, consistent with finding 10 yesterday).</t>
     </r>
+  </si>
+  <si>
+    <t>2011_occupation_msoa.csv (data);
+2021_occupation_msoa.csv (data);
+lsoa11_to_msoa11.csv (output);</t>
   </si>
 </sst>
 </file>
@@ -3104,13 +3104,13 @@
         <v>46200</v>
       </c>
       <c r="D42" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="F42" s="3" t="s">
         <v>168</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>169</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>166</v>

</xml_diff>

<commit_message>
Completed eda 5 - comparison with Yee&Dennett's attribute detection
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9F536B-7829-F843-B84E-22FAA23BE9AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81BC5CBB-FFFE-7848-B661-6E6639260F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1735,13 +1735,76 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>, consistent with finding 10 yesterday).</t>
+      <t xml:space="preserve">, consistent with finding 10 yesterday).
+3. Comparing with Yee's detection: a) </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Majority of MSOAs are labelled as "Stable"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in Yee's work, no matter which typology. b) Among gentrification labels, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>majority MSOAs were "Cascade-led"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, while there is a tiny subsets of MSOAs were "Counter-led". </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Yee's labels and my typology don't influence, mirror, or align with each other in any meaningful way</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
     </r>
   </si>
   <si>
     <t>2011_occupation_msoa.csv (data);
 2021_occupation_msoa.csv (data);
-lsoa11_to_msoa11.csv (output);</t>
+lsoa11_to_msoa11.csv (output);
+eda_5_yee_msoa_comparison_20260627.ipynb;
+yee_cascade_comparison_20260627.csv (output);</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Completed eda 6 - comparison wit occupational ascent analysis (Duncan)
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81BC5CBB-FFFE-7848-B661-6E6639260F07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21FA31F1-E717-5240-AB33-DB25F1FBE0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1796,7 +1796,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>.</t>
+      <t>.
+4. Comparing with occupational ascent analysis: a) Occupational ascent are independent from cascade typology.</t>
     </r>
   </si>
   <si>
@@ -1804,7 +1805,8 @@
 2021_occupation_msoa.csv (data);
 lsoa11_to_msoa11.csv (output);
 eda_5_yee_msoa_comparison_20260627.ipynb;
-yee_cascade_comparison_20260627.csv (output);</t>
+yee_cascade_comparison_20260627.csv (output);
+occupation_comparison_20260627.csv (output)</t>
   </si>
 </sst>
 </file>
@@ -3162,7 +3164,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" ht="221" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>46200</v>
       </c>

</xml_diff>

<commit_message>
Update eda 4 part 3a and part 4
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21FA31F1-E717-5240-AB33-DB25F1FBE0D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DDA9C7-F8F0-4040-9C8B-C4EC879A2E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="176">
   <si>
     <t>Date</t>
   </si>
@@ -1801,12 +1801,123 @@
     </r>
   </si>
   <si>
+    <r>
+      <t>Both results from comaprison work mean there is no actual correlation between attribute-detection and my flow typology. i.e. Knowing a place is cascade experiencing implies nothing about gentrification status. Why?
+But</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> if we know a place has gentrification label, we can have more confidence to know it is experiencing cascade, though there are small possibilities of counter flows as well.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Why?
+</t>
+    </r>
+  </si>
+  <si>
     <t>2011_occupation_msoa.csv (data);
 2021_occupation_msoa.csv (data);
 lsoa11_to_msoa11.csv (output);
 eda_5_yee_msoa_comparison_20260627.ipynb;
 yee_cascade_comparison_20260627.csv (output);
-occupation_comparison_20260627.csv (output)</t>
+occupation_comparison_20260627.csv (output);
+eda_6_occupational_comparison_20260627.ipynb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_4_rerun_compare_natioanl_frame_and_london_only__20260625.ipynb;
+eda_5_yee_msoa_comparison_20260627.ipynb;
+eda_6_occupational_comparison_20260627.ipynb
+</t>
+  </si>
+  <si>
+    <t>1. Confirm Duncan's occupation classification;
+2. Spatial distribution of flow typology shift, especially about where are typology -&gt; cascade-led; where are typology -&gt; counter-led</t>
+  </si>
+  <si>
+    <t>eda_5_yee_msoa_comparison_20260627.ipynb;
+eda_6_occupational_comparison_20260627.ipynb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. How to understand the difference between 2 arms of the cascade churn - inflow from wealthier and outflow to poorer? The shares changed  over the decade.
+</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cascade-flow detection is decoupled from the IMD-improvement, which defines attribute-gentrification, and it does NOT track improvement the way GEN does</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. -- EDA 5 --&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Cascade is mainly about neighbourhood restructuring, not strongly correlated with gentrification as we expected before</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Flow is independent from demographic composition.;
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cascade flow is NOT the engine of IMD-measured gentrification. Cascade does NOT reinforce gentrification</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. - EDA 5
+2. Duncan's article confirmed important outer London social changes, especially in Bromley, Barnet, etc, places identified in my study (among top12 cascade dominated places by 2021).</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3168,22 +3279,46 @@
       <c r="A42" s="1">
         <v>46200</v>
       </c>
+      <c r="B42" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>171</v>
+      </c>
       <c r="D42" s="3" t="s">
         <v>167</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>168</v>
       </c>
+      <c r="G42" s="3" t="s">
+        <v>169</v>
+      </c>
       <c r="H42" s="3" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>46201</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
completed eda 5 and eda 6
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DDA9C7-F8F0-4040-9C8B-C4EC879A2E2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9EB713-C38E-334B-ACF3-D825B0507484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="178">
   <si>
     <t>Date</t>
   </si>
@@ -749,55 +749,6 @@
 ks101ew_lsoa_2011_allengland.csv
 data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb
 </t>
-  </si>
-  <si>
-    <r>
-      <t>Outside London is a big proportion missed so far, need to be analysed in the next step. -- High priority.
-Compare with attribute-based detections (Duncan Smith's work- professional change 2011-2021), there are some flagged areas in attribute-based dection, but shown as "Lateral" in current typology.
-1. London-relative analysis captures intra-urban restructuring. The national-frame analysis checks whether accounting for London's exchange with the rest of England changes the structural pattern. The two analyses are complementray. (</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>London-relative result first, then national-frame extension to show if cascade/counter balance shifts</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">).
-2. London is more deprived than England on average. Comparing London and national wide, the internal deprivation hierarchy is preserved, but only the absolute position changes.
-3. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Most flows from outside London into London would register as `Inflow_Wealthier` (cascade direction), and most flows from London to outside will register as `Outflow_Wealthier`</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
   </si>
   <si>
     <t>Data preprocess;
@@ -1694,114 +1645,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">0. Net Counter = Outflow_Wealthier - Inflow_Poorer, so positive Net_Counter means more people move to wealthier areas than people moving from poorer areas. Need to watch out the logic.
-1. For replication of Duncan's work, the ONS table page for the 2021 NS-SeC (TS062) explicitly warns it's not comparable with the 2011 Census because the classifications in the occupation variable have changed. So we need to replicate the usage of SOC major group (1 Managers/Directors, 2 Professional, 3 Associate Professional), rather than NS-SeC.
-2. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>2021 cascade-dominance shift is not tracking attribute-gentrification, it's flow restructuring [exodus]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (from </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>uncorrelation between affluent share change and IMD change in occupational analysis comparison</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, consistent with finding 10 yesterday).
-3. Comparing with Yee's detection: a) </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Majority of MSOAs are labelled as "Stable"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> in Yee's work, no matter which typology. b) Among gentrification labels, </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>majority MSOAs were "Cascade-led"</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, while there is a tiny subsets of MSOAs were "Counter-led". </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Yee's labels and my typology don't influence, mirror, or align with each other in any meaningful way</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.
-4. Comparing with occupational ascent analysis: a) Occupational ascent are independent from cascade typology.</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t>Both results from comaprison work mean there is no actual correlation between attribute-detection and my flow typology. i.e. Knowing a place is cascade experiencing implies nothing about gentrification status. Why?
 But</t>
     </r>
@@ -1850,32 +1693,10 @@
 eda_6_occupational_comparison_20260627.ipynb</t>
   </si>
   <si>
-    <t xml:space="preserve">1. How to understand the difference between 2 arms of the cascade churn - inflow from wealthier and outflow to poorer? The shares changed  over the decade.
-</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Cascade-flow detection is decoupled from the IMD-improvement, which defines attribute-gentrification, and it does NOT track improvement the way GEN does</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">. -- EDA 5 --&gt; </t>
+    <r>
+      <t xml:space="preserve">0. Net Counter = Outflow_Wealthier - Inflow_Poorer, so positive Net_Counter means more people move to wealthier areas than people moving from poorer areas. Need to watch out the logic.
+1. For replication of Duncan's work, the ONS table page for the 2021 NS-SeC (TS062) explicitly warns it's not comparable with the 2011 Census because the classifications in the occupation variable have changed. So we need to replicate the usage of SOC major group (1 Managers/Directors, 2 Professional, 3 Associate Professional), rather than NS-SeC.
+2. </t>
     </r>
     <r>
       <rPr>
@@ -1884,6 +1705,119 @@
         <color rgb="FFFF0000"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
+      <t>2021 cascade-dominance shift is not tracking attribute-gentrification, it's flow restructuring [exodus]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (from </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>uncorrelation between affluent share change and IMD change in occupational analysis comparison</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, consistent with finding 10 yesterday).
+3. Comparing with occupational ascent analysis: a) Occupational ascent are independent from cascade typology.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">refined map figs;
+</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. How to understand the difference between 2 arms of the cascade churn - inflow from wealthier and outflow to poorer? The shares changed  over the decade.
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Should we widen "gentrifying" as "gentrifying + incumbent upgrade"?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> I think no, since we focus on migration, incumbent mean not relocate.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>2021 flow patterns are consistent with COVID-era suburbanisation, but we're not sure if caused by it</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cascade-flow detection is decoupled from the IMD-improvement, which defines attribute-gentrification, and it does NOT track improvement the way GEN does</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. -- EDA 5 --&gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
       <t>Cascade is mainly about neighbourhood restructuring, not strongly correlated with gentrification as we expected before</t>
     </r>
     <r>
@@ -1894,7 +1828,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">. Flow is independent from demographic composition.;
+      <t xml:space="preserve">.
 2. </t>
     </r>
     <r>
@@ -1905,6 +1839,86 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
+      <t xml:space="preserve">Yee-GEN tracks IMD improvement, directionally as a gentrification signal,  while flow typology does NOT. We can't treat cascade flow as a proxy for IMD-defined gentrification. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Though</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Both attribute and flow typologies are weak predictors of IMD change</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.; -- EDA 5
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Yee's gentrifying areas, where they carry a flow signature, lean cascade and essentially never counter</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. Yee's method and my method </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>agree</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> where and when classic inner-Londonn gentrification was happening. -- EDA 5
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Cascade flow is NOT the engine of IMD-measured gentrification. Cascade does NOT reinforce gentrification</t>
     </r>
     <r>
@@ -1915,8 +1929,80 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>. - EDA 5
+      <t xml:space="preserve">. - EDA 5
+4. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>The affluent-in-movement signal moved from inner to outer boroughs across the decade.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Inner London cascade collapsed. Outer London absorbed and generated cascade. ~85% (166/195) of outer MSOAs supplies Cascade-led. -- EDA5
 2. Duncan's article confirmed important outer London social changes, especially in Bromley, Barnet, etc, places identified in my study (among top12 cascade dominated places by 2021).</t>
+    </r>
+  </si>
+  <si>
+    <t>Catch up with Adam.</t>
+  </si>
+  <si>
+    <r>
+      <t>Compare with attribute-based detections (Duncan Smith's work- professional change 2011-2021), there are some flagged areas in attribute-based dection, but shown as "Lateral" in current typology.
+1. London-relative analysis captures intra-urban restructuring. The national-frame analysis checks whether accounting for London's exchange with the rest of England changes the structural pattern. The two analyses are complementray. (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>London-relative result first, then national-frame extension to show if cascade/counter balance shifts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">).
+2. London is more deprived than England on average. Comparing London and national wide, the internal deprivation hierarchy is preserved, but only the absolute position changes.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Most flows from outside London into London would register as `Inflow_Wealthier` (cascade direction), and most flows from London to outside will register as `Outflow_Wealthier`</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
     </r>
   </si>
 </sst>
@@ -3145,7 +3231,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="306" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" ht="170" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>46195</v>
       </c>
@@ -3153,7 +3239,7 @@
         <v>136</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>137</v>
@@ -3162,7 +3248,7 @@
         <v>139</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>140</v>
+        <v>177</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>135</v>
@@ -3171,30 +3257,30 @@
         <v>134</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="323" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" ht="221" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>46196</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="E38" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="F38" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="G38" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="G38" s="3" t="s">
+      <c r="H38" s="3" t="s">
         <v>147</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
@@ -3202,51 +3288,51 @@
         <v>46197</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C39" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G39" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D39" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="F39" s="3" t="s">
+      <c r="H39" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="G39" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="306" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="1:8" ht="272" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>46198</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C40" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="E40" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G40" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="E40" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G40" s="3" t="s">
+      <c r="H40" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
@@ -3257,25 +3343,25 @@
         <v>10</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D41" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>165</v>
-      </c>
       <c r="G41" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="H41" s="3" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="221" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="1:8" ht="204" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>46200</v>
       </c>
@@ -3283,25 +3369,25 @@
         <v>3</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D42" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G42" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E42" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>169</v>
-      </c>
       <c r="H42" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="272" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>46201</v>
       </c>
@@ -3309,16 +3395,22 @@
         <v>10</v>
       </c>
       <c r="C43" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>172</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>175</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>174</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added progress summary file
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9EB713-C38E-334B-ACF3-D825B0507484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDA2D5A-9E66-074B-9174-969B990202A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1740,10 +1740,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">refined map figs;
-</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1. How to understand the difference between 2 arms of the cascade churn - inflow from wealthier and outflow to poorer? The shares changed  over the decade.
 2. </t>
@@ -2004,6 +2000,11 @@
       </rPr>
       <t>.</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">refined map figs;
+Progress_Summary_20260628.md (meet-prep).
+</t>
   </si>
 </sst>
 </file>
@@ -3248,7 +3249,7 @@
         <v>139</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>135</v>
@@ -3401,16 +3402,16 @@
         <v>170</v>
       </c>
       <c r="E43" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="G43" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="H43" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Completed progress summary file
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BDA2D5A-9E66-074B-9174-969B990202A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BC3D2BD-2E72-4B49-A267-D43C88B3E295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1741,50 +1741,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">1. How to understand the difference between 2 arms of the cascade churn - inflow from wealthier and outflow to poorer? The shares changed  over the decade.
-2. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>Should we widen "gentrifying" as "gentrifying + incumbent upgrade"?</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> I think no, since we focus on migration, incumbent mean not relocate.
-3. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>2021 flow patterns are consistent with COVID-era suburbanisation, but we're not sure if caused by it</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">.
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">1. </t>
     </r>
     <r>
@@ -2005,6 +1961,50 @@
     <t xml:space="preserve">refined map figs;
 Progress_Summary_20260628.md (meet-prep).
 </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. How to understand the difference between 2 arms of the cascade churn - inflow from wealthier and outflow to poorer? The shares changed  over the decade.
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Should we widen "gentrifying" as "gentrifying + incumbent upgrade"?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> I think no, since we focus on migration, incumbent mean not relocate.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>2021 flow patterns are consistent with COVID-era suburbanisation, but we're not sure if caused by it</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">. I think we should decribe this in the discussion part.
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3249,7 +3249,7 @@
         <v>139</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>135</v>
@@ -3402,16 +3402,16 @@
         <v>170</v>
       </c>
       <c r="E43" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="G43" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="H43" s="2" t="s">
         <v>174</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
added and updated eda 7 about case studies
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F76D544-5608-AB4E-AA2A-80BCFA0D8BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B1B4B3-6D75-E746-ADD4-E8B3F736E117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -1685,10 +1685,6 @@
 </t>
   </si>
   <si>
-    <t>1. Confirm Duncan's occupation classification;
-2. Spatial distribution of flow typology shift, especially about where are typology -&gt; cascade-led; where are typology -&gt; counter-led</t>
-  </si>
-  <si>
     <t>eda_5_yee_msoa_comparison_20260627.ipynb;
 eda_6_occupational_comparison_20260627.ipynb</t>
   </si>
@@ -1791,11 +1787,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">refined map figs;
-Progress_Summary_20260628.md (meet-prep).
-</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1. How to understand the difference between 2 arms of the cascade churn - inflow from wealthier and outflow to poorer? The shares changed  over the decade.
 2. </t>
@@ -2006,6 +1997,20 @@
 5. Duncan's article confirmed important outer London social changes, especially in Bromley, Barnet, etc, places identified in my study (among top12 cascade dominated places by 2021).
 6. Duncan also pointed out his data could not tell whether gentrification processes displace lower income people in London.</t>
     </r>
+  </si>
+  <si>
+    <t>1. Confirm Duncan's occupation classification;
+2. Spatial distribution of flow typology shift, especially about where are typology -&gt; cascade-led; where are typology -&gt; counter-led;
+3. Special study cases to show city-wide counter dominance by 2021.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">refined map figs;
+Progress_Summary_20260628.md (meet-prep);
+fig_case_A_persistent_cascade.png;
+fig_case_B_cascade_to_counter.png;
+fig_case_C_exodus.png;
+eda_7_case_study_202060628.ipynb
+</t>
   </si>
 </sst>
 </file>
@@ -3250,7 +3255,7 @@
         <v>139</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>135</v>
@@ -3380,7 +3385,7 @@
         <v>168</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>167</v>
@@ -3397,22 +3402,22 @@
         <v>10</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="E43" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F43" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="F43" s="3" t="s">
-        <v>177</v>
-      </c>
       <c r="G43" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
meeting - research logbook updated
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06B1B4B3-6D75-E746-ADD4-E8B3F736E117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6455056-697A-C342-A756-70819B9106B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="181">
   <si>
     <t>Date</t>
   </si>
@@ -1573,27 +1573,7 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-1. Add borough names on the map for better readability
-2. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>Confirm with Duncan about the SOC major groups he used</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
+1. Add borough names on the map for better readability</t>
     </r>
   </si>
   <si>
@@ -1641,32 +1621,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>"</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Both results from comaprison work mean there is no actual correlation between attribute-detection and my flow typology. i.e. Knowing a place is cascade experiencing implies nothing about gentrification status. Why?
-But</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF00B0F0"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve"> if we know a place has gentrification label, we can have more confidence to know it is experiencing cascade, though there are small possibilities of counter flows as well.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Why?
-</t>
     </r>
   </si>
   <si>
@@ -2011,6 +1965,42 @@
 fig_case_C_exodus.png;
 eda_7_case_study_202060628.ipynb
 </t>
+  </si>
+  <si>
+    <r>
+      <t>Both results from comaprison work mean there is no actual correlation between attribute-detection and my flow typology. i.e. Knowing a place is cascade experiencing implies nothing about gentrification status. Why?
+But</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve"> if we know a place has gentrification label, we can have more confidence to know it is experiencing cascade, though there are small possibilities of counter flows as well.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Why? --- Not really, they're two different mechanisms.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Everything we worked so far.</t>
+  </si>
+  <si>
+    <t>Why both Yee's method and my method can not strongly explain IMD changes? Is that because we just analysed IMD percentile changes?
+Should we use other data or references?</t>
+  </si>
+  <si>
+    <t>Prepare presentation slides for the mini conference.</t>
   </si>
 </sst>
 </file>
@@ -2483,7 +2473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="1" bestFit="1" customWidth="1"/>
@@ -3255,7 +3245,7 @@
         <v>139</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>135</v>
@@ -3376,19 +3366,19 @@
         <v>3</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>166</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>165</v>
@@ -3402,27 +3392,48 @@
         <v>10</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D43" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>177</v>
-      </c>
       <c r="F43" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>46202</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
@@ -3433,6 +3444,41 @@
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>46204</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
+        <v>46206</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
+        <v>46208</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
+        <v>46209</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" s="1">
+        <v>46210</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" s="1">
+        <v>46211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added presentation slides for mini-conference, still updating...
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6455056-697A-C342-A756-70819B9106B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCA7143-8A06-FF4B-B3BA-6AE6CA4DFDF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="188">
   <si>
     <t>Date</t>
   </si>
@@ -2001,6 +2001,113 @@
   </si>
   <si>
     <t>Prepare presentation slides for the mini conference.</t>
+  </si>
+  <si>
+    <t>Mini conference presentation</t>
+  </si>
+  <si>
+    <t>How to present the methodology and findings in a coherent and logic way?</t>
+  </si>
+  <si>
+    <t>presentation slide v1</t>
+  </si>
+  <si>
+    <t>presentation slide v2</t>
+  </si>
+  <si>
+    <t>presentation slide v3, v4</t>
+  </si>
+  <si>
+    <t>presentation slide v5, v6</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Outer London became more socio-economically advantaged. (revisit from Duncan's article)
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Cascade_Dominance</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is designed as a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>measure of directional replacement pressure</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, not direct replacement of people. We're asking "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>How much a neighbourhood's turnover is organised by the deprivation hierarchy?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">" Defensible arguments from this neighbourhood migration study can be "population turnover is dominated by exchanges with less deprived neighbourhoods." Cascade_Dominance as migration data, is lack of causal meaning to represent displacement, which can't be inferred from the flow pattern alone.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Cascade_Dominance provides an ecological indicator of hierarchical neighbourhood replacement. A high value indicates that population turnover is predominatly driven by exchanges with less deprived neighbourhoods rather than counter-hierarchical movements. While this does not identify the socioeconomic characteristics of individual movers or establish displacement, it quantifies the extent to which neighbourhood restructuring follows a deprivation-ordered hierarchy.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+4. We're safe to state "hierarchical population turnover", "social-spatial restructuring", "neighbourhoods re-sorting". And we should avoid to say "displacement", "household replacement".</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2098,8 +2205,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2476,1018 +2586,1085 @@
   <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="37.1640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="75.1640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="89.5" style="2" customWidth="1"/>
-    <col min="6" max="6" width="151.33203125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="59.83203125" style="2" customWidth="1"/>
-    <col min="8" max="8" width="63" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="10.83203125" style="2"/>
+    <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="37.1640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="75.1640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="89.5" style="3" customWidth="1"/>
+    <col min="6" max="6" width="151.33203125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="59.83203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="63" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45796</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45797</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45798</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45799</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="4" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45800</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="4" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
+      <c r="A9" s="2">
         <v>45801</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A10" s="1">
+      <c r="A10" s="2">
         <v>45802</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="4" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="323" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
+      <c r="A11" s="2">
         <v>46168</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="5" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:8" s="6" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="7" t="s">
+      <c r="G12" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="8" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="4"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
+      <c r="A13" s="5"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="10" t="s">
+      <c r="D14" s="7"/>
+      <c r="E14" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="6"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="10" t="s">
+      <c r="F14" s="7"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="11" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="8"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="10"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="1">
+      <c r="A16" s="2">
         <v>46174</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="11" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="G17" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="H17" s="10"/>
+      <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="8"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A19" s="1">
+      <c r="A19" s="2">
         <v>46177</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="H19" s="4" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="1">
+      <c r="A20" s="2">
         <v>46178</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="11" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
+      <c r="A21" s="2">
         <v>46179</v>
       </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="2" t="s">
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="10"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="1">
+      <c r="A22" s="2">
         <v>46180</v>
       </c>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="2" t="s">
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="10"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="1">
+      <c r="A23" s="2">
         <v>46181</v>
       </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="2" t="s">
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="10"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
     </row>
     <row r="24" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
+      <c r="A24" s="2">
         <v>46182</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G24" s="3" t="s">
+      <c r="G24" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="H24" s="4" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
+      <c r="A25" s="2">
         <v>46183</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="E25" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G25" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H25" s="11" t="s">
+      <c r="H25" s="12" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A26" s="1">
+      <c r="A26" s="2">
         <v>46184</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="3" t="s">
+      <c r="B26" s="11"/>
+      <c r="C26" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="G26" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="H26" s="11"/>
+      <c r="H26" s="12"/>
     </row>
     <row r="27" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A27" s="1">
+      <c r="A27" s="2">
         <v>46185</v>
       </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="3" t="s">
+      <c r="B27" s="11"/>
+      <c r="C27" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="E27" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G27" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="H27" s="11"/>
+      <c r="H27" s="12"/>
     </row>
     <row r="28" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A28" s="1">
+      <c r="A28" s="2">
         <v>46186</v>
       </c>
-      <c r="B28" s="10"/>
-      <c r="C28" s="3" t="s">
+      <c r="B28" s="11"/>
+      <c r="C28" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="E28" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="G28" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="H28" s="11"/>
+      <c r="H28" s="12"/>
     </row>
     <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
+      <c r="A29" s="2">
         <v>46187</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="3" t="s">
+      <c r="B29" s="11"/>
+      <c r="C29" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="E29" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F29" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="G29" s="3" t="s">
+      <c r="G29" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="H29" s="3" t="s">
+      <c r="H29" s="4" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
+      <c r="A30" s="2">
         <v>46188</v>
       </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="3" t="s">
+      <c r="B30" s="11"/>
+      <c r="C30" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H30" s="11" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="1">
+      <c r="A31" s="2">
         <v>46189</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="F31" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="G31" s="12" t="s">
+      <c r="G31" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="H31" s="10"/>
+      <c r="H31" s="11"/>
     </row>
     <row r="32" spans="1:8" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="1">
+      <c r="A32" s="2">
         <v>46190</v>
       </c>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="2" t="s">
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E32" s="10"/>
-      <c r="F32" s="11"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
     </row>
     <row r="33" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="1">
+      <c r="A33" s="2">
         <v>46191</v>
       </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="11" t="s">
+      <c r="B33" s="11"/>
+      <c r="C33" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="D33" s="11" t="s">
+      <c r="D33" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="E33" s="11" t="s">
+      <c r="E33" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="F33" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G33" s="11" t="s">
+      <c r="G33" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="H33" s="11" t="s">
+      <c r="H33" s="12" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="1">
+      <c r="A34" s="2">
         <v>46192</v>
       </c>
-      <c r="B34" s="10"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
     </row>
     <row r="35" spans="1:8" ht="268" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="1">
+      <c r="A35" s="2">
         <v>46193</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="3" t="s">
+      <c r="B35" s="11"/>
+      <c r="C35" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="E35" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="G35" s="13" t="s">
+      <c r="G35" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="H35" s="3" t="s">
+      <c r="H35" s="4" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="1">
+      <c r="A36" s="2">
         <v>46194</v>
       </c>
-      <c r="C36" s="3" t="s">
+      <c r="C36" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="E36" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F36" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="G36" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="H36" s="3" t="s">
+      <c r="H36" s="4" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="170" x14ac:dyDescent="0.2">
-      <c r="A37" s="1">
+      <c r="A37" s="2">
         <v>46195</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E37" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="G37" s="3" t="s">
+      <c r="G37" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="H37" s="3" t="s">
+      <c r="H37" s="4" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="221" x14ac:dyDescent="0.2">
-      <c r="A38" s="1">
+      <c r="A38" s="2">
         <v>46196</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E38" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="F38" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="G38" s="3" t="s">
+      <c r="G38" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="H38" s="3" t="s">
+      <c r="H38" s="4" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A39" s="1">
+      <c r="A39" s="2">
         <v>46197</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E39" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="F39" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="G39" s="3" t="s">
+      <c r="G39" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="H39" s="3" t="s">
+      <c r="H39" s="4" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="272" x14ac:dyDescent="0.2">
-      <c r="A40" s="1">
+      <c r="A40" s="2">
         <v>46198</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="B40" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="C40" s="3" t="s">
+      <c r="C40" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="E40" s="3" t="s">
+      <c r="E40" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="F40" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="G40" s="3" t="s">
+      <c r="G40" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="H40" s="3" t="s">
+      <c r="H40" s="4" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A41" s="1">
+      <c r="A41" s="2">
         <v>46199</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="D41" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="E41" s="3" t="s">
+      <c r="E41" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="F41" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="G41" s="3" t="s">
+      <c r="G41" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="H41" s="3" t="s">
+      <c r="H41" s="4" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="204" x14ac:dyDescent="0.2">
-      <c r="A42" s="1">
+      <c r="A42" s="2">
         <v>46200</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C42" s="3" t="s">
+      <c r="C42" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="F42" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="G42" s="3" t="s">
+      <c r="G42" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="H42" s="3" t="s">
+      <c r="H42" s="4" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="306" x14ac:dyDescent="0.2">
-      <c r="A43" s="1">
+      <c r="A43" s="2">
         <v>46201</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="C43" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="4" t="s">
         <v>175</v>
       </c>
-      <c r="E43" s="3" t="s">
+      <c r="E43" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="G43" s="3" t="s">
+      <c r="G43" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="H43" s="3" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A44" s="1">
+      <c r="A44" s="2">
         <v>46202</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="C44" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="D44" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="E44" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="F44" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G44" s="3" t="s">
+      <c r="G44" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="H44" s="8" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" s="1">
+      <c r="A45" s="2">
         <v>46203</v>
       </c>
+      <c r="B45" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G45" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H45" s="8"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="1">
+      <c r="A46" s="2">
         <v>46204</v>
       </c>
+      <c r="B46" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D46" s="8"/>
+      <c r="E46" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" s="1">
+      <c r="A47" s="2">
         <v>46205</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" s="1">
+      <c r="B47" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D47" s="8"/>
+      <c r="E47" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8"/>
+    </row>
+    <row r="48" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+      <c r="A48" s="2">
         <v>46206</v>
       </c>
+      <c r="B48" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="D48" s="8"/>
+      <c r="E48" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" s="1">
+      <c r="A49" s="2">
         <v>46207</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" s="1">
+      <c r="A50" s="2">
         <v>46208</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" s="1">
+      <c r="A51" s="2">
         <v>46209</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" s="1">
+      <c r="A52" s="2">
         <v>46210</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" s="1">
+      <c r="A53" s="2">
         <v>46211</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="44">
     <mergeCell ref="H30:H32"/>
     <mergeCell ref="H33:H34"/>
     <mergeCell ref="E33:E34"/>
     <mergeCell ref="F33:F34"/>
     <mergeCell ref="G33:G34"/>
+    <mergeCell ref="D45:D48"/>
+    <mergeCell ref="G45:G48"/>
+    <mergeCell ref="H44:H48"/>
     <mergeCell ref="C33:C34"/>
     <mergeCell ref="D33:D34"/>
     <mergeCell ref="B25:B30"/>

</xml_diff>

<commit_message>
Updated eda 7 - case studies visualisation refined
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCA7143-8A06-FF4B-B3BA-6AE6CA4DFDF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9856981C-282C-F64B-BB9B-1453D159F03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="193">
   <si>
     <t>Date</t>
   </si>
@@ -2108,6 +2108,29 @@
       <t xml:space="preserve">
 4. We're safe to state "hierarchical population turnover", "social-spatial restructuring", "neighbourhoods re-sorting". And we should avoid to say "displacement", "household replacement".</t>
     </r>
+  </si>
+  <si>
+    <t>1. Ruth stated “The upward swing in standards of living, moreover, not only contributes to all the other space requirements, but also increase those individual households, and helps to create more households.” Would this be consistent with the current counter dominated pattern.
+2. So far, from description of "displacement" by Ruth, "displacement" seems always coexist with "replacement", and plus the identifications between who replace who.</t>
+  </si>
+  <si>
+    <t>Literature review;
+Communication;
+EDA</t>
+  </si>
+  <si>
+    <t>Mini conference presentation;
+Ruth_Glass-Aspect_od_change (reading-archive-repo)；
+Conceptual_framework_v6_202060704;
+eda_7_refined_case_study_202060704.ipynb</t>
+  </si>
+  <si>
+    <t>Ruth_Glass-Aspect_od_change (reading-archive-repo);
+eda_7_refined_case_study_202060704.ipynb</t>
+  </si>
+  <si>
+    <t>How to understand displacement and restructuring, in the context of gentrification?
+How to make case study visualisation better to the audience? To make it easier to read and understand without the full load of contexts.</t>
   </si>
 </sst>
 </file>
@@ -3630,27 +3653,42 @@
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" ht="102" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>46207</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B49" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46208</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>46209</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>46210</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>46211</v>
       </c>

</xml_diff>

<commit_message>
eda 8, after eda 7 - case locator map to visualise locations of each flow mechanisms on the map
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9856981C-282C-F64B-BB9B-1453D159F03B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9927A05F-2795-2B4F-85CC-5A3700E6EFFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2119,18 +2119,20 @@
 EDA</t>
   </si>
   <si>
+    <t>How to understand displacement and restructuring, in the context of gentrification?
+How to make case study visualisation better to the audience? To make it easier to read and understand without the full load of contexts.</t>
+  </si>
+  <si>
+    <t>Ruth_Glass-Aspect_od_change (reading-archive-repo);
+eda_7_refined_case_study_202060704.ipynb;
+eda_8_case_locator_map_20260704.ipynb</t>
+  </si>
+  <si>
     <t>Mini conference presentation;
 Ruth_Glass-Aspect_od_change (reading-archive-repo)；
 Conceptual_framework_v6_202060704;
-eda_7_refined_case_study_202060704.ipynb</t>
-  </si>
-  <si>
-    <t>Ruth_Glass-Aspect_od_change (reading-archive-repo);
-eda_7_refined_case_study_202060704.ipynb</t>
-  </si>
-  <si>
-    <t>How to understand displacement and restructuring, in the context of gentrification?
-How to make case study visualisation better to the audience? To make it easier to read and understand without the full load of contexts.</t>
+eda_7_refined_case_study_202060704.ipynb;
+eda_8_case_locator_map_20260704.ipynb</t>
   </si>
 </sst>
 </file>
@@ -2611,7 +2613,7 @@
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="37.1640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" style="3" customWidth="1"/>
     <col min="4" max="4" width="75.1640625" style="3" customWidth="1"/>
     <col min="5" max="5" width="89.5" style="3" customWidth="1"/>
     <col min="6" max="6" width="151.33203125" style="3" customWidth="1"/>
@@ -3653,7 +3655,7 @@
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
     </row>
-    <row r="49" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" ht="119" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>46207</v>
       </c>
@@ -3661,10 +3663,10 @@
         <v>189</v>
       </c>
       <c r="C49" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D49" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>192</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>191</v>

</xml_diff>

<commit_message>
Updated eda 8 - temporal comparison with cascade churn 2 flows split analysis
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6732E173-29BB-554C-8BC1-6852987D1372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84FD1580-ECEF-804F-8046-755D9B48DF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="195">
   <si>
     <t>Date</t>
   </si>
@@ -2115,10 +2115,6 @@
 EDA</t>
   </si>
   <si>
-    <t>How to understand displacement and restructuring, in the context of gentrification?
-How to make case study visualisation better to the audience? To make it easier to read and understand without the full load of contexts.</t>
-  </si>
-  <si>
     <t>Ruth_Glass-Aspect_od_change (reading-archive-repo);
 eda_7_refined_case_study_202060704.ipynb;
 eda_8_case_locator_map_20260704.ipynb</t>
@@ -2134,6 +2130,18 @@
     <t xml:space="preserve">1. Ruth stated “The upward swing in standards of living, moreover, not only contributes to all the other space requirements, but also increase those individual households, and helps to create more households.” Would this be consistent with the current counter dominated pattern.
 2. So far, from description of "displacement" by Ruth, "displacement" seems always coexist with "replacement", and plus the identifications between who replace who.
 ** Found a cute interactive visualisation website to present migration analysis: https://worldmigrationreport.iom.int/msite/wmr-2024-interactive/ </t>
+  </si>
+  <si>
+    <t>How to understand displacement and restructuring, in the context of gentrification?
+How to make case study visualisation better to the audience? To make it easier to read and understand without the full load of contexts.
+Is exodus cascade the same as the outflow-driven cascade?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In eda 8, after temporal comparison fig, map small multiple versions with the same pair but faceted by ring - inner and outer with the count table
+</t>
+  </si>
+  <si>
+    <t>Is exodus the same as outflow-driven? I think yes in this study so far.</t>
   </si>
 </sst>
 </file>
@@ -3656,7 +3664,7 @@
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
     </row>
-    <row r="49" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>46207</v>
       </c>
@@ -3664,34 +3672,40 @@
         <v>188</v>
       </c>
       <c r="C49" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="F49" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G49" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46208</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>46209</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>46210</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>46211</v>
       </c>

</xml_diff>

<commit_message>
Updated eda 8 - need further split about the outflow-driven to show exodus
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84FD1580-ECEF-804F-8046-755D9B48DF8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB57FDAB-A400-3841-9DB6-51E8B6623CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2127,21 +2127,66 @@
 eda_8_case_locator_map_20260704.ipynb</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Ruth stated “The upward swing in standards of living, moreover, not only contributes to all the other space requirements, but also increase those individual households, and helps to create more households.” Would this be consistent with the current counter dominated pattern.
-2. So far, from description of "displacement" by Ruth, "displacement" seems always coexist with "replacement", and plus the identifications between who replace who.
-** Found a cute interactive visualisation website to present migration analysis: https://worldmigrationreport.iom.int/msite/wmr-2024-interactive/ </t>
-  </si>
-  <si>
     <t>How to understand displacement and restructuring, in the context of gentrification?
 How to make case study visualisation better to the audience? To make it easier to read and understand without the full load of contexts.
 Is exodus cascade the same as the outflow-driven cascade?</t>
   </si>
   <si>
-    <t xml:space="preserve">In eda 8, after temporal comparison fig, map small multiple versions with the same pair but faceted by ring - inner and outer with the count table
+    <r>
+      <t xml:space="preserve">Is exodus the same as outflow-driven? </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Exodus means not frame robust AND outflow-led cascade</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">;
 </t>
-  </si>
-  <si>
-    <t>Is exodus the same as outflow-driven? I think yes in this study so far.</t>
+    </r>
+  </si>
+  <si>
+    <t>In eda 8, after temporal comparison fig, map small multiple versions with the same pair but faceted by ring - inner and outer with the count table
+Still in eda 8, carefully treat "exodus" for both 2011 and 2021. Exodus exists after comparing between frames over periods!! How to present "exodus" and "outflow-driven" on both 2011 and 2021?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Ruth stated “The upward swing in standards of living, moreover, not only contributes to all the other space requirements, but also increase those individual households, and helps to create more households.” Would this be consistent with the current counter dominated pattern.
+2. So far, from description of "displacement" by Ruth, "displacement" seems always coexist with "replacement", and plus the identifications between who replace who.
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Cascade-led can be split into inflow-driven-cascade and outflow-driven-cascade, outflow-driven-cascade can then been split as external-dominated or not</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+** Found a cute interactive visualisation website to present migration analysis: https://worldmigrationreport.iom.int/msite/wmr-2024-interactive/ </t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3664,7 +3709,7 @@
       <c r="G48" s="8"/>
       <c r="H48" s="8"/>
     </row>
-    <row r="49" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" ht="136" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>46207</v>
       </c>
@@ -3675,16 +3720,16 @@
         <v>190</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>189</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="G49" s="3" t="s">
         <v>194</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>192</v>
       </c>
       <c r="H49" s="4" t="s">
         <v>193</v>

</xml_diff>

<commit_message>
Added eda 9 time-symmetric tree code file
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB57FDAB-A400-3841-9DB6-51E8B6623CED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C825833-212A-174C-AA6B-0F5D3BB20E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="198">
   <si>
     <t>Date</t>
   </si>
@@ -2158,10 +2158,6 @@
     </r>
   </si>
   <si>
-    <t>In eda 8, after temporal comparison fig, map small multiple versions with the same pair but faceted by ring - inner and outer with the count table
-Still in eda 8, carefully treat "exodus" for both 2011 and 2021. Exodus exists after comparing between frames over periods!! How to present "exodus" and "outflow-driven" on both 2011 and 2021?</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">1. Ruth stated “The upward swing in standards of living, moreover, not only contributes to all the other space requirements, but also increase those individual households, and helps to create more households.” Would this be consistent with the current counter dominated pattern.
 2. So far, from description of "displacement" by Ruth, "displacement" seems always coexist with "replacement", and plus the identifications between who replace who.
@@ -2187,6 +2183,45 @@
       <t xml:space="preserve">.
 ** Found a cute interactive visualisation website to present migration analysis: https://worldmigrationreport.iom.int/msite/wmr-2024-interactive/ </t>
     </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">In eda 8, after temporal comparison fig, map small multiple versions with the same pair but faceted by ring - inner and outer with the count table
+Still in eda 8, carefully treat "exodus" for both 2011 and 2021. Exodus exists after comparing between frames over periods!! </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>further split outflow-driven-cascade as exodus (yellow colour) or not</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>eda_9;
+(refined)eda_7;
+(refined) eda_8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
+</t>
+  </si>
+  <si>
+    <t>eda_9;
+(refined)eda_7;
+(refined) eda_8_v2</t>
   </si>
 </sst>
 </file>
@@ -3726,18 +3761,27 @@
         <v>189</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>192</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46208</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added eda 10 - rerun case locator map with tree mechanism
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C825833-212A-174C-AA6B-0F5D3BB20E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821A28F8-7A43-354F-9DB7-F794A249703D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2212,16 +2212,20 @@
   <si>
     <t>eda_9;
 (refined)eda_7;
-(refined) eda_8</t>
+(refined) eda_8_v2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_9;
+(refined)eda_7;
+eda_10 [refined eda 8];
+eda9_mechanism_tree_20260705.csv (outputs);
+</t>
   </si>
   <si>
     <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
+- Threshold of cascade inflow share
+- Threshold of outflow external share
 </t>
-  </si>
-  <si>
-    <t>eda_9;
-(refined)eda_7;
-(refined) eda_8_v2</t>
   </si>
 </sst>
 </file>
@@ -3770,18 +3774,18 @@
         <v>194</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46208</v>
       </c>
       <c r="C50" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D50" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="E50" s="4" t="s">
         <v>196</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added eda 11 - updated eda 7 alluvial plots after eda 9 new mechanisms; a new mechanism D after splitting outflow regarding external outflow shares
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{821A28F8-7A43-354F-9DB7-F794A249703D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2296D4B6-9BCE-5C41-968C-C9EE49176B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2215,16 +2215,16 @@
 (refined) eda_8_v2</t>
   </si>
   <si>
-    <t xml:space="preserve">eda_9;
-(refined)eda_7;
-eda_10 [refined eda 8];
-eda9_mechanism_tree_20260705.csv (outputs);
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
 - Threshold of cascade inflow share
 - Threshold of outflow external share
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_9;
+eda_10 [refined eda 8];
+eda_11_from_eda7_new_case_study__new_mechanism_20260705.ipynb;
+eda9_mechanism_tree_20260705.csv (outputs);
 </t>
   </si>
 </sst>
@@ -3782,10 +3782,10 @@
         <v>195</v>
       </c>
       <c r="D50" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E50" s="4" t="s">
         <v>197</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
debug eda 4 - some code cell logic issues - have sorted
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2296D4B6-9BCE-5C41-968C-C9EE49176B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39C18145-C38F-CD47-B32F-1529FB3A177F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="202">
   <si>
     <t>Date</t>
   </si>
@@ -2158,6 +2158,63 @@
     </r>
   </si>
   <si>
+    <t>eda_9_mechanism_tree_20260705.ipynb;
+eda_9_threshold_justification_mechanism_tree_20260705.ipynb;
+eda_10 [refined eda 8];
+eda_11_from_eda7_new_case_study__new_mechanism_20260705.ipynb;
+eda9_mechanism_tree_20260705.csv (outputs);
+new figs in case_study after running eda 9-11.</t>
+  </si>
+  <si>
+    <t>Case study files:
+- eda_9;
+- (refined)eda_7;
+- (refined) eda_8_v2</t>
+  </si>
+  <si>
+    <t>EDA;
+Communication</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>In eda 8, after temporal comparison fig, map small multiple versions with the same pair but faceted by ring - inner and outer with the count table</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Still in eda 8, carefully treat "exodus" for both 2011 and 2021. Exodus exists after comparing between frames over periods!! </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>further split outflow-driven-cascade as exodus (yellow colour) or not</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">1. Ruth stated “The upward swing in standards of living, moreover, not only contributes to all the other space requirements, but also increase those individual households, and helps to create more households.” Would this be consistent with the current counter dominated pattern.
 2. So far, from description of "displacement" by Ruth, "displacement" seems always coexist with "replacement", and plus the identifications between who replace who.
@@ -2167,7 +2224,7 @@
       <rPr>
         <b/>
         <sz val="12"/>
-        <color rgb="FFFF0000"/>
+        <color theme="1"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
       <t>Cascade-led can be split into inflow-driven-cascade and outflow-driven-cascade, outflow-driven-cascade can then been split as external-dominated or not</t>
@@ -2185,47 +2242,81 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">In eda 8, after temporal comparison fig, map small multiple versions with the same pair but faceted by ring - inner and outer with the count table
-Still in eda 8, carefully treat "exodus" for both 2011 and 2021. Exodus exists after comparing between frames over periods!! </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>further split outflow-driven-cascade as exodus (yellow colour) or not</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.</t>
-    </r>
-  </si>
-  <si>
-    <t>eda_9;
-(refined)eda_7;
-(refined) eda_8_v2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
+    <t>1. We built a new tree mechanism to explore interesting cases of cascade-led MSOAs. --- EDA 9
+2. Even splitting cascade-led as inflow-driven and outflow-drive, we can still split further with outflow-driven. Outflow-driven can be either external as majority or not. External as majority increased quite much by 2021. --- EDA 9&amp;11</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Do we need to test the external share in inflow-driven? Or we can just defend this with no great external share inflow, so it would not affect much? (we split inflow-driven with typology robustness, but split outflow with external shares); -- though ppl would ask why use different conditions? We use different because we observed comparison results with Yee's labels. Would this comparison waved after this mechanism?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
 - Threshold of cascade inflow share
 - Threshold of outflow external share
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">eda_9;
-eda_10 [refined eda 8];
-eda_11_from_eda7_new_case_study__new_mechanism_20260705.ipynb;
-eda9_mechanism_tree_20260705.csv (outputs);
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">;
 </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Debug eda 4 rerun!
+compute how many outflow-led MSOAs change category between Frame B and Frame C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Rerun Yee's comparison with new tree mechanisms.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2323,7 +2414,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2365,6 +2456,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3765,27 +3859,39 @@
         <v>189</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>192</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="136" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46208</v>
       </c>
+      <c r="B50" s="4" t="s">
+        <v>195</v>
+      </c>
       <c r="C50" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>197</v>
+        <v>193</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G50" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated eda 9b - robustness of frames B&C between inflow-led and outflow-led
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B8980B-2469-BC4A-AF83-5E8F49E087F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC88FB7-3143-3B4E-8713-3272B27EC9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2158,12 +2158,6 @@
     </r>
   </si>
   <si>
-    <t>Case study files:
-- eda_9;
-- (refined)eda_7;
-- (refined) eda_8_v2</t>
-  </si>
-  <si>
     <t>EDA;
 Communication</t>
   </si>
@@ -2234,77 +2228,37 @@
     </r>
   </si>
   <si>
-    <t>1. We built a new tree mechanism to explore interesting cases of cascade-led MSOAs. --- EDA 9
-2. Even splitting cascade-led as inflow-driven and outflow-drive, we can still split further with outflow-driven. Outflow-driven can be either external as majority or not. External as majority increased quite much by 2021. --- EDA 9&amp;11</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Do we need to test the external share in inflow-driven? Or we can just defend this with no great external share inflow, so it would not affect much? (we split inflow-driven with typology robustness, but split outflow with external shares); -- though ppl would ask why use different conditions? We use different because we observed comparison results with Yee's labels. Would this comparison waved after this mechanism?</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+    <t xml:space="preserve">1. We built a new tree mechanism to explore interesting cases of cascade-led MSOAs. --- EDA 9
+2. Even splitting cascade-led as inflow-driven and outflow-drive, we can still split further with outflow-driven. Outflow-driven can be either external as majority or not. External as majority increased quite much by 2021. --- EDA 9&amp;11;
+3. External/Internal-driven outflow is actually partially because of frame switch. --- EDA 9 4i;
+</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Debug eda 4 rerun! (done)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
       </rPr>
       <t xml:space="preserve">
 </t>
     </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
-- Threshold of cascade inflow share
-- Threshold of outflow external share
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">;
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>Debug eda 4 rerun! (done)</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve">
-compute how many outflow-led MSOAs change category between Frame B and Frame C</t>
+      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C (done)</t>
     </r>
     <r>
       <rPr>
@@ -2325,7 +2279,58 @@
 eda_11_from_eda7_new_case_study__new_mechanism_20260705.ipynb;
 eda9_mechanism_tree_20260705.csv (outputs);
 new figs in case_study after running eda 9-11;
-eda_4_rerun_compare_national_frame_and_london_only_FIXED_20260705.ipynb</t>
+eda_4_rerun_compare_national_frame_and_london_only_FIXED_20260705.ipynb;
+eda_12_redo_yee_leaf_corroboration_20260705.ipynb</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
+- Threshold of cascade inflow share
+- Threshold of outflow external share
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;
+Redo corroboration with Yee's labels using new leaves;</t>
+    </r>
+  </si>
+  <si>
+    <t>Case study files:
+- eda_9;
+- (refined)eda_7;
+- (refined) eda_8_v2;
+eda 12 (redo Yee's label comparison).</t>
+  </si>
+  <si>
+    <r>
+      <t>Do we need to test the external share in inflow-driven? Or we can just defend this with no great external share inflow, so it would not affect much? (we split inflow-driven with typology robustness, but split outflow with external shares); -- though ppl would ask why use different conditions? We use different because we observed comparison results with Yee's labels. Would this comparison waved after this mechanism? (solved - methodology v9 draft subtab)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -3868,13 +3873,13 @@
         <v>189</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G49" s="4" t="s">
         <v>192</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="136" x14ac:dyDescent="0.2">
@@ -3882,25 +3887,25 @@
         <v>46208</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="D50" s="4" t="s">
         <v>199</v>
       </c>
       <c r="E50" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="G50" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="H50" s="4" t="s">
         <v>197</v>
-      </c>
-      <c r="G50" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated eda 12 - geunine persistent set is different from eda 11
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC88FB7-3143-3B4E-8713-3272B27EC9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B3F783-48B5-A048-8431-31043FEA123F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2228,51 +2228,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">1. We built a new tree mechanism to explore interesting cases of cascade-led MSOAs. --- EDA 9
-2. Even splitting cascade-led as inflow-driven and outflow-drive, we can still split further with outflow-driven. Outflow-driven can be either external as majority or not. External as majority increased quite much by 2021. --- EDA 9&amp;11;
-3. External/Internal-driven outflow is actually partially because of frame switch. --- EDA 9 4i;
-</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>Debug eda 4 rerun! (done)</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C (done)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Rerun Yee's comparison with new tree mechanisms.</t>
-    </r>
-  </si>
-  <si>
     <t>eda_9_mechanism_tree_20260705.ipynb;
 eda_9_threshold_justification_mechanism_tree_20260705.ipynb;
 eda_10 [refined eda 8];
@@ -2330,6 +2285,78 @@
       </rPr>
       <t xml:space="preserve">
 </t>
+    </r>
+  </si>
+  <si>
+    <t>1. We built a new tree mechanism to explore interesting cases of cascade-led MSOAs. --- EDA 9
+2. Even splitting cascade-led as inflow-driven and outflow-drive, we can still split further with outflow-driven. Outflow-driven can be either external as majority or not. External as majority increased quite much by 2021. --- EDA 9&amp;11;
+3. External/Internal-driven outflow is actually partially because of frame switch. --- EDA 9 4i;
+4. GEN labels does NOT concentrate with inflow-driven cascade, strong signal is with outflow-internal. Not overlapped as expected with genuine cascade. Then decomposition with GEN class3 subtype. --- EDA 12</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Debug eda 4 rerun! (done)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C (done)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Rerun Yee's comparison with new tree mechanisms. --- </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">supGEN and MainGen about Camden and Tower Hamlets are not both inflow-driven -- eda 11 case roster? </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>I doubt this is because eda 12 concludes with the whole borough, eda 11 picked 2 specific MSOAs in those 2 boroughs.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> EDA 12 genuine persistent set does not contain eda 11 cases fig a!!</t>
     </r>
   </si>
 </sst>
@@ -3882,7 +3909,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" ht="170" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46208</v>
       </c>
@@ -3890,22 +3917,22 @@
         <v>193</v>
       </c>
       <c r="C50" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="F50" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="G50" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="E50" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F50" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="G50" s="15" t="s">
+      <c r="H50" s="4" t="s">
         <v>201</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added presentation slides v7
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B3F783-48B5-A048-8431-31043FEA123F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E496439-8C59-7941-93E7-8F7815B8BD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2228,6 +2228,128 @@
     </r>
   </si>
   <si>
+    <r>
+      <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
+- Threshold of cascade inflow share
+- Threshold of outflow external share
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;
+Redo corroboration with Yee's labels using new leaves;</t>
+    </r>
+  </si>
+  <si>
+    <t>Case study files:
+- eda_9;
+- (refined)eda_7;
+- (refined) eda_8_v2;
+eda 12 (redo Yee's label comparison).</t>
+  </si>
+  <si>
+    <r>
+      <t>Do we need to test the external share in inflow-driven? Or we can just defend this with no great external share inflow, so it would not affect much? (we split inflow-driven with typology robustness, but split outflow with external shares); -- though ppl would ask why use different conditions? We use different because we observed comparison results with Yee's labels. Would this comparison waved after this mechanism? (solved - methodology v9 draft subtab)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>1. We built a new tree mechanism to explore interesting cases of cascade-led MSOAs. --- EDA 9
+2. Even splitting cascade-led as inflow-driven and outflow-drive, we can still split further with outflow-driven. Outflow-driven can be either external as majority or not. External as majority increased quite much by 2021. --- EDA 9&amp;11;
+3. External/Internal-driven outflow is actually partially because of frame switch. --- EDA 9 4i;
+4. GEN labels does NOT concentrate with inflow-driven cascade, strong signal is with outflow-internal. Not overlapped as expected with genuine cascade. Then decomposition with GEN class3 subtype. --- EDA 12</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>Debug eda 4 rerun! (done)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C (done)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Rerun Yee's comparison with new tree mechanisms. --- </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t xml:space="preserve">supGEN and MainGen about Camden and Tower Hamlets are not both inflow-driven -- eda 11 case roster? </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
+      <t>I doubt this is because eda 12 concludes with the whole borough, eda 11 picked 2 specific MSOAs in those 2 boroughs.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> EDA 12 genuine persistent set does not contain eda 11 cases fig a!! but they match with eda 10 map!</t>
+    </r>
+  </si>
+  <si>
     <t>eda_9_mechanism_tree_20260705.ipynb;
 eda_9_threshold_justification_mechanism_tree_20260705.ipynb;
 eda_10 [refined eda 8];
@@ -2235,129 +2357,8 @@
 eda9_mechanism_tree_20260705.csv (outputs);
 new figs in case_study after running eda 9-11;
 eda_4_rerun_compare_national_frame_and_london_only_FIXED_20260705.ipynb;
-eda_12_redo_yee_leaf_corroboration_20260705.ipynb</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Logic of the time-symmetric tree of cascade-led flow mechanisms;
-- Threshold of cascade inflow share
-- Threshold of outflow external share
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>;
-Redo corroboration with Yee's labels using new leaves;</t>
-    </r>
-  </si>
-  <si>
-    <t>Case study files:
-- eda_9;
-- (refined)eda_7;
-- (refined) eda_8_v2;
-eda 12 (redo Yee's label comparison).</t>
-  </si>
-  <si>
-    <r>
-      <t>Do we need to test the external share in inflow-driven? Or we can just defend this with no great external share inflow, so it would not affect much? (we split inflow-driven with typology robustness, but split outflow with external shares); -- though ppl would ask why use different conditions? We use different because we observed comparison results with Yee's labels. Would this comparison waved after this mechanism? (solved - methodology v9 draft subtab)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <t>1. We built a new tree mechanism to explore interesting cases of cascade-led MSOAs. --- EDA 9
-2. Even splitting cascade-led as inflow-driven and outflow-drive, we can still split further with outflow-driven. Outflow-driven can be either external as majority or not. External as majority increased quite much by 2021. --- EDA 9&amp;11;
-3. External/Internal-driven outflow is actually partially because of frame switch. --- EDA 9 4i;
-4. GEN labels does NOT concentrate with inflow-driven cascade, strong signal is with outflow-internal. Not overlapped as expected with genuine cascade. Then decomposition with GEN class3 subtype. --- EDA 12</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>Debug eda 4 rerun! (done)</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>compute how many outflow-led MSOAs change category between Frame B and Frame C (done)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Rerun Yee's comparison with new tree mechanisms. --- </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t xml:space="preserve">supGEN and MainGen about Camden and Tower Hamlets are not both inflow-driven -- eda 11 case roster? </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>I doubt this is because eda 12 concludes with the whole borough, eda 11 picked 2 specific MSOAs in those 2 boroughs.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> EDA 12 genuine persistent set does not contain eda 11 cases fig a!!</t>
-    </r>
+eda_12_redo_yee_leaf_corroboration_20260705.ipynb;
+Flow_Gentrification_Deck_v7_20260705.pptx</t>
   </si>
 </sst>
 </file>
@@ -3909,7 +3910,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" ht="187" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46208</v>
       </c>
@@ -3917,22 +3918,22 @@
         <v>193</v>
       </c>
       <c r="C50" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="G50" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="D50" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="F50" s="4" t="s">
+      <c r="H50" s="4" t="s">
         <v>200</v>
-      </c>
-      <c r="G50" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added eda 3b - same-decile outflow test & presentation scripts
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E496439-8C59-7941-93E7-8F7815B8BD77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF5B174-72FE-6941-86DA-F9F0A49D9881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="211">
   <si>
     <t>Date</t>
   </si>
@@ -2360,13 +2360,48 @@
 eda_12_redo_yee_leaf_corroboration_20260705.ipynb;
 Flow_Gentrification_Deck_v7_20260705.pptx</t>
   </si>
+  <si>
+    <t>eda 12;
+presentation slides</t>
+  </si>
+  <si>
+    <t>How to understand the comaprison with Yee's labels</t>
+  </si>
+  <si>
+    <t>deck_v8;
+deck_v9;
+eda_12_v3</t>
+  </si>
+  <si>
+    <t>all conclusions in deck v9 and eda_12_v3</t>
+  </si>
+  <si>
+    <t>How to understand the overlap in labels from LSOA to MSOA? There are some MSOAs with multuple GEN subtype labels.</t>
+  </si>
+  <si>
+    <t>How to make presentation clear to audience?
+Does the same decile migration change current results a lot?</t>
+  </si>
+  <si>
+    <t>eda_3b_cascade_definition_sensitivity_20260708.ipynb;
+presentation scripts</t>
+  </si>
+  <si>
+    <t>eda_3b_cascade_definition_sensitivity_20260708.ipynb;
+eda_3b_cascade_definition_sensitivity_summary.csv;
+presentation script</t>
+  </si>
+  <si>
+    <t>Same-decile out-moves are ~0.4× the to-poorer arm and ~17% of all out-migration.
+If adding same-decile moves to "outflow to poorer-or-same" against the mirror "inflow from poorer-or-same" — cascade-led barely moves. We also considered the same-decile moves in the typology alreadly as they are considered in the metric ofcross-decile shares.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -2461,7 +2496,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2470,22 +2505,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2494,14 +2520,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2837,7 +2872,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -3059,7 +3094,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="323" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" ht="221" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>46168</v>
       </c>
@@ -3085,71 +3120,71 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="6" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:8" s="5" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="B12" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="G12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="H12" s="10" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="5"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="11" t="s">
+      <c r="D14" s="14"/>
+      <c r="E14" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="7"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="11" t="s">
+      <c r="F14" s="14"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="9"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="11"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
@@ -3173,43 +3208,43 @@
       <c r="G16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="8" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B17" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="11" t="s">
+      <c r="D17" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="H17" s="11"/>
+      <c r="H17" s="8"/>
     </row>
     <row r="18" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="9"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
     </row>
     <row r="19" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
@@ -3241,25 +3276,25 @@
       <c r="A20" s="2">
         <v>46178</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="9" t="s">
         <v>87</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H20" s="8" t="s">
         <v>23</v>
       </c>
     </row>
@@ -3267,43 +3302,43 @@
       <c r="A21" s="2">
         <v>46179</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="9"/>
       <c r="E21" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>46180</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="12"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="9"/>
       <c r="E22" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>46181</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="12"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="9"/>
       <c r="E23" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
     </row>
     <row r="24" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
@@ -3335,7 +3370,7 @@
       <c r="A25" s="2">
         <v>46183</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="8" t="s">
         <v>93</v>
       </c>
       <c r="C25" s="4" t="s">
@@ -3353,7 +3388,7 @@
       <c r="G25" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H25" s="12" t="s">
+      <c r="H25" s="9" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3361,7 +3396,7 @@
       <c r="A26" s="2">
         <v>46184</v>
       </c>
-      <c r="B26" s="11"/>
+      <c r="B26" s="8"/>
       <c r="C26" s="4" t="s">
         <v>95</v>
       </c>
@@ -3377,13 +3412,13 @@
       <c r="G26" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="H26" s="12"/>
-    </row>
-    <row r="27" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="H26" s="9"/>
+    </row>
+    <row r="27" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>46185</v>
       </c>
-      <c r="B27" s="11"/>
+      <c r="B27" s="8"/>
       <c r="C27" s="4" t="s">
         <v>101</v>
       </c>
@@ -3399,13 +3434,13 @@
       <c r="G27" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="H27" s="12"/>
+      <c r="H27" s="9"/>
     </row>
     <row r="28" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>46186</v>
       </c>
-      <c r="B28" s="11"/>
+      <c r="B28" s="8"/>
       <c r="C28" s="4" t="s">
         <v>104</v>
       </c>
@@ -3421,13 +3456,13 @@
       <c r="G28" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="H28" s="12"/>
+      <c r="H28" s="9"/>
     </row>
     <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>46187</v>
       </c>
-      <c r="B29" s="11"/>
+      <c r="B29" s="8"/>
       <c r="C29" s="4" t="s">
         <v>107</v>
       </c>
@@ -3451,7 +3486,7 @@
       <c r="A30" s="2">
         <v>46188</v>
       </c>
-      <c r="B30" s="11"/>
+      <c r="B30" s="8"/>
       <c r="C30" s="4" t="s">
         <v>113</v>
       </c>
@@ -3467,7 +3502,7 @@
       <c r="G30" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H30" s="11" t="s">
+      <c r="H30" s="8" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3475,61 +3510,61 @@
       <c r="A31" s="2">
         <v>46189</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="8" t="s">
         <v>119</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="F31" s="12" t="s">
+      <c r="F31" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="G31" s="13" t="s">
+      <c r="G31" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="H31" s="11"/>
+      <c r="H31" s="8"/>
     </row>
     <row r="32" spans="1:8" ht="92" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>46190</v>
       </c>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
       <c r="D32" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E32" s="11"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
     </row>
     <row r="33" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>46191</v>
       </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="12" t="s">
+      <c r="B33" s="8"/>
+      <c r="C33" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="D33" s="12" t="s">
+      <c r="D33" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="E33" s="12" t="s">
+      <c r="E33" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="F33" s="12" t="s">
+      <c r="F33" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G33" s="12" t="s">
+      <c r="G33" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="H33" s="12" t="s">
+      <c r="H33" s="9" t="s">
         <v>9</v>
       </c>
     </row>
@@ -3537,19 +3572,19 @@
       <c r="A34" s="2">
         <v>46192</v>
       </c>
-      <c r="B34" s="11"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
     </row>
     <row r="35" spans="1:8" ht="268" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>46193</v>
       </c>
-      <c r="B35" s="11"/>
+      <c r="B35" s="8"/>
       <c r="C35" s="4" t="s">
         <v>124</v>
       </c>
@@ -3562,7 +3597,7 @@
       <c r="F35" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="G35" s="14" t="s">
+      <c r="G35" s="6" t="s">
         <v>138</v>
       </c>
       <c r="H35" s="4" t="s">
@@ -3644,7 +3679,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>46197</v>
       </c>
@@ -3696,7 +3731,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>46199</v>
       </c>
@@ -3796,7 +3831,7 @@
       <c r="G44" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="H44" s="8" t="s">
+      <c r="H44" s="10" t="s">
         <v>180</v>
       </c>
     </row>
@@ -3810,7 +3845,7 @@
       <c r="C45" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D45" s="10" t="s">
         <v>182</v>
       </c>
       <c r="E45" s="3" t="s">
@@ -3819,10 +3854,10 @@
       <c r="F45" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G45" s="8" t="s">
+      <c r="G45" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="H45" s="8"/>
+      <c r="H45" s="10"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
@@ -3834,15 +3869,15 @@
       <c r="C46" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D46" s="8"/>
+      <c r="D46" s="10"/>
       <c r="E46" s="3" t="s">
         <v>184</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="10"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
@@ -3854,15 +3889,15 @@
       <c r="C47" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D47" s="8"/>
+      <c r="D47" s="10"/>
       <c r="E47" s="3" t="s">
         <v>185</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
     </row>
     <row r="48" spans="1:8" ht="204" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
@@ -3874,15 +3909,15 @@
       <c r="C48" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D48" s="8"/>
+      <c r="D48" s="10"/>
       <c r="E48" s="3" t="s">
         <v>186</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G48" s="8"/>
-      <c r="H48" s="8"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
     </row>
     <row r="49" spans="1:8" ht="136" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
@@ -3929,62 +3964,81 @@
       <c r="F50" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="G50" s="15" t="s">
+      <c r="G50" s="7" t="s">
         <v>198</v>
       </c>
       <c r="H50" s="4" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>46209</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B51" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
-        <v>46210</v>
+        <v>46211</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
-        <v>46211</v>
+        <v>46212</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" s="2">
+        <v>46213</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" s="2">
+        <v>46214</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" s="2">
+        <v>46215</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="H30:H32"/>
-    <mergeCell ref="H33:H34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="D45:D48"/>
-    <mergeCell ref="G45:G48"/>
-    <mergeCell ref="H44:H48"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="B25:B30"/>
-    <mergeCell ref="H25:H28"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="D20:D23"/>
-    <mergeCell ref="F20:F23"/>
-    <mergeCell ref="G20:G23"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H16:H18"/>
     <mergeCell ref="H12:H13"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="B14:B15"/>
@@ -3997,6 +4051,38 @@
     <mergeCell ref="C12:C13"/>
     <mergeCell ref="A12:A13"/>
     <mergeCell ref="E12:E13"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H16:H18"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="C20:C23"/>
+    <mergeCell ref="D20:D23"/>
+    <mergeCell ref="F20:F23"/>
+    <mergeCell ref="G20:G23"/>
+    <mergeCell ref="B25:B30"/>
+    <mergeCell ref="H25:H28"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="D45:D48"/>
+    <mergeCell ref="G45:G48"/>
+    <mergeCell ref="H44:H48"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="H30:H32"/>
+    <mergeCell ref="H33:H34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="G33:G34"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update eda 10 - correct Kingston MSOA name
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{926376AD-3F46-2845-88E8-72B2AE156C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873A4F55-7F95-4F4D-99BE-44515F2196BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="221">
   <si>
     <t>Date</t>
   </si>
@@ -2421,6 +2421,14 @@
   </si>
   <si>
     <t>Waiting feedbacks from mini conference.</t>
+  </si>
+  <si>
+    <t>Communication;
+EDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">eda_10fixed_case_locator_map_labels_20260714.ipynb;
+</t>
   </si>
 </sst>
 </file>
@@ -2899,7 +2907,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4149,6 +4157,17 @@
       </c>
       <c r="H56" s="3" t="s">
         <v>218</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A57" s="2">
+        <v>46217</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added addtional analysis about migration distance in data preprocess rerun file
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873A4F55-7F95-4F4D-99BE-44515F2196BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55619A6-38F6-9947-97C5-5AEBC399440F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="226">
   <si>
     <t>Date</t>
   </si>
@@ -2429,6 +2429,23 @@
   <si>
     <t xml:space="preserve">eda_10fixed_case_locator_map_labels_20260714.ipynb;
 </t>
+  </si>
+  <si>
+    <t>dissertation draft</t>
+  </si>
+  <si>
+    <t>eda_10fixed_case_locator_map_labels_20260714.ipynb;
+dissertation drafts</t>
+  </si>
+  <si>
+    <t>Does the "Flow" has been considered as share in the analysis so far? --- Yes, CDS and cascade dominance can defend for this.</t>
+  </si>
+  <si>
+    <t>How to trim current drafts? We need to set a story line as a core and use results and code files we have to enrich this sotry;
+We have so much can tell, but not very clear as a story line.</t>
+  </si>
+  <si>
+    <t>Refine dissertation draft.</t>
   </si>
 </sst>
 </file>
@@ -4159,15 +4176,30 @@
         <v>218</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>46217</v>
       </c>
       <c r="B57" s="4" t="s">
         <v>219</v>
       </c>
+      <c r="C57" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>221</v>
+      </c>
       <c r="E57" s="4" t="s">
         <v>220</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added dissertation skeleton & methodology v11 (unfinished, leaving from 3.5 untouched)
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B55619A6-38F6-9947-97C5-5AEBC399440F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DCF190C-3988-FE40-AC6B-CF64C370A8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
+    <workbookView xWindow="15100" yWindow="660" windowWidth="15140" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="235">
   <si>
     <t>Date</t>
   </si>
@@ -2427,8 +2427,7 @@
 EDA</t>
   </si>
   <si>
-    <t xml:space="preserve">eda_10fixed_case_locator_map_labels_20260714.ipynb;
-</t>
+    <t>eda_10fixed_case_locator_map_labels_20260714.ipynb</t>
   </si>
   <si>
     <t>dissertation draft</t>
@@ -2446,6 +2445,41 @@
   </si>
   <si>
     <t>Refine dissertation draft.</t>
+  </si>
+  <si>
+    <t>data_preprocess_rerun_national_frame_20260625.ipynb;
+dissertation drafts</t>
+  </si>
+  <si>
+    <t>How to understand the deprivation pocket, though this is out of the scope of this study;
+A quick check on the migration distance - would it be a big factor in migration itself?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Additional check in data preprocess rerun file;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. People don't hop across London. Every hierarchy-crossing moves have medians around 4km, meaning people cross deciles without going far. [For deprivation pocket], it's only possible to change decile within 4km because London's deprivation surface is a fine-grained mosaic where different deciles sit close together.
+2. Downward moves are consistently shorter than upward moves.
+</t>
+  </si>
+  <si>
+    <t>Communication;
+Dissertation draft</t>
+  </si>
+  <si>
+    <t>Dissertation skeleton - google drive</t>
+  </si>
+  <si>
+    <t>How to structure the whole dissertation?
+The main argument is gentrification theories often assume a migration cascade mechanism — wealthier households moving into neighbourhoods while poorer households move out — but this process is usually inferred from changes in neighbourhood attributes rather than observed directly through migration flows. Therefore, the dissertation treats the cascade mechanism itself as a hypothesis to be tested using census origin-destination migration data and a deprivation hierarchy framework.</t>
+  </si>
+  <si>
+    <t>Waiting feedback from Adam about the strcture and feedbacks from mini conference</t>
+  </si>
+  <si>
+    <t>Dissertation skeleton in google drive;
+mehtodology-v11</t>
   </si>
 </sst>
 </file>
@@ -2924,7 +2958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4200,6 +4234,55 @@
       </c>
       <c r="H57" s="3" t="s">
         <v>225</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A58" s="2">
+        <v>46218</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+      <c r="A59" s="2">
+        <v>46219</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finished methodology draft - v12
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DCF190C-3988-FE40-AC6B-CF64C370A8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1BB128-B3A9-B042-B855-4FC9764F1FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15100" yWindow="660" windowWidth="15140" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
+    <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="242">
   <si>
     <t>Date</t>
   </si>
@@ -2480,6 +2480,28 @@
   <si>
     <t>Dissertation skeleton in google drive;
 mehtodology-v11</t>
+  </si>
+  <si>
+    <t>mehtodology-v12</t>
+  </si>
+  <si>
+    <t>(remove all discussion and results part from the methodology chapter! Keep everything methodological-driven!)</t>
+  </si>
+  <si>
+    <t>Keep refining methodology - v12</t>
+  </si>
+  <si>
+    <t>Start drafting results chapter and discussion chapter.</t>
+  </si>
+  <si>
+    <t>Dissertation draft</t>
+  </si>
+  <si>
+    <t>methodology v12 - google drive</t>
+  </si>
+  <si>
+    <t>Can't use any validation, we're comparing between methods;
+Keep the methdology chapter purely methodological-driven.</t>
   </si>
 </sst>
 </file>
@@ -2958,7 +2980,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4283,6 +4305,58 @@
       </c>
       <c r="H59" s="4" t="s">
         <v>233</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" s="2">
+        <v>46221</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A61" s="2">
+        <v>46222</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added eda 13 - use new measure to compare with Yee and Dennett's class-3 subtypes
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1BB128-B3A9-B042-B855-4FC9764F1FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7352F87-CBB0-C94A-978E-655F9E668EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="249">
   <si>
     <t>Date</t>
   </si>
@@ -2502,6 +2502,54 @@
   <si>
     <t>Can't use any validation, we're comparing between methods;
 Keep the methdology chapter purely methodological-driven.</t>
+  </si>
+  <si>
+    <t>methodology v13 - google drive;
+result v4 - google drive</t>
+  </si>
+  <si>
+    <t>result v3 - google drive</t>
+  </si>
+  <si>
+    <t>result v3</t>
+  </si>
+  <si>
+    <t>Start drafting discussion chapter.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Revised core argument: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">A coarse cascade classification does not provide a universal measure of gentrification because the same flow signature can arise from different mechanisms;
+reference-frame and mechanism decomposition are therefore necessary before comparison with attribute-based gentrification measures.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Quit the "lift" measure in eda 12, use direct proportion and counting measures to compare with class-3 subtype.</t>
+    </r>
+  </si>
+  <si>
+    <t>methodology v13 - google drive;
+result v4 - google drive;
+eda 13 (scripts)</t>
+  </si>
+  <si>
+    <t>How to make the comparison between mechanisms and class-3 subtype eaiser to understand;
+Need to adjust the measures of this subtype comparison.</t>
   </si>
 </sst>
 </file>
@@ -2980,7 +3028,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4303,7 +4351,7 @@
       <c r="G59" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H59" s="4" t="s">
+      <c r="H59" s="6" t="s">
         <v>233</v>
       </c>
     </row>
@@ -4357,6 +4405,84 @@
       </c>
       <c r="H61" s="3" t="s">
         <v>238</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" s="2">
+        <v>46223</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" s="2">
+        <v>46224</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A64" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added literature review drafts
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7352F87-CBB0-C94A-978E-655F9E668EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5192C52B-5CBA-6A40-9176-55268CC34E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="254">
   <si>
     <t>Date</t>
   </si>
@@ -2504,10 +2504,6 @@
 Keep the methdology chapter purely methodological-driven.</t>
   </si>
   <si>
-    <t>methodology v13 - google drive;
-result v4 - google drive</t>
-  </si>
-  <si>
     <t>result v3 - google drive</t>
   </si>
   <si>
@@ -2550,6 +2546,26 @@
   <si>
     <t>How to make the comparison between mechanisms and class-3 subtype eaiser to understand;
 Need to adjust the measures of this subtype comparison.</t>
+  </si>
+  <si>
+    <t>discussion v2 - google drive</t>
+  </si>
+  <si>
+    <t>Drafting lit review chapter.</t>
+  </si>
+  <si>
+    <t>discussion v2 - google drive -- 1985 words</t>
+  </si>
+  <si>
+    <t>methodology v13 - google drive -- 2560 words;
+result v4 - google drive -- 1861 words</t>
+  </si>
+  <si>
+    <t>literature-review v3;
+literature-review v4  - google drive -- 1777 words</t>
+  </si>
+  <si>
+    <t>Need more referernces to support some arguments and statements</t>
   </si>
 </sst>
 </file>
@@ -3028,7 +3044,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4415,13 +4431,13 @@
         <v>239</v>
       </c>
       <c r="C62" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E62" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="F62" s="3" t="s">
         <v>23</v>
@@ -4441,13 +4457,13 @@
         <v>239</v>
       </c>
       <c r="C63" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E63" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>244</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>23</v>
@@ -4467,22 +4483,74 @@
         <v>239</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="D64" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A65" s="2">
+        <v>46227</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E65" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="E64" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="F64" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="G64" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H64" s="3" t="s">
-        <v>245</v>
+      <c r="F65" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A66" s="2">
+        <v>46228</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refined drafts for lit review, methodology, results, and discussion
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5192C52B-5CBA-6A40-9176-55268CC34E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38933F61-F1ED-F047-81DF-C4A8928BB518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="257">
   <si>
     <t>Date</t>
   </si>
@@ -2566,6 +2566,22 @@
   </si>
   <si>
     <t>Need more referernces to support some arguments and statements</t>
+  </si>
+  <si>
+    <t>cascade_dominance symmetric bandwidth sensitivity check.</t>
+  </si>
+  <si>
+    <t>literature-review v5  - google drive -- 1849 words;
+methodology v14 - google drive -- 2844 words;
+results v5 - google drive -- 2132 words;
+discussion v3 - google drive -- 2051 words</t>
+  </si>
+  <si>
+    <t>literature-review v5  - google drive -- 1849 words;
+methodology v14 - google drive -- 2844 words;
+results v5 - google drive -- 2132 words;
+discussion v3 - google drive -- 2051 words
+8876 in total</t>
   </si>
 </sst>
 </file>
@@ -3044,7 +3060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4551,6 +4567,32 @@
       </c>
       <c r="H66" s="3" t="s">
         <v>253</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+      <c r="A67" s="2">
+        <v>46229</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E67" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
meeting prep doc - 20260726
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38933F61-F1ED-F047-81DF-C4A8928BB518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE51B2D-6A6C-B649-B638-459D4728B97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2574,14 +2574,15 @@
     <t>literature-review v5  - google drive -- 1849 words;
 methodology v14 - google drive -- 2844 words;
 results v5 - google drive -- 2132 words;
-discussion v3 - google drive -- 2051 words</t>
+discussion v3 - google drive -- 2051 words
+8876 in total</t>
   </si>
   <si>
     <t>literature-review v5  - google drive -- 1849 words;
 methodology v14 - google drive -- 2844 words;
 results v5 - google drive -- 2132 words;
-discussion v3 - google drive -- 2051 words
-8876 in total</t>
+discussion v3 - google drive -- 2051 words;
+Dissertation_Roadmap_Meeting_20260727.docx</t>
   </si>
 </sst>
 </file>
@@ -4577,13 +4578,13 @@
         <v>239</v>
       </c>
       <c r="C67" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E67" s="4" t="s">
         <v>256</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>255</v>
       </c>
       <c r="F67" s="3" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
Refine and update locator map - colour and case studies - eda 10 and eda 12
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE51B2D-6A6C-B649-B638-459D4728B97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B03036-4033-304D-9986-3FF98662BD32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="263">
   <si>
     <t>Date</t>
   </si>
@@ -2583,6 +2583,33 @@
 results v5 - google drive -- 2132 words;
 discussion v3 - google drive -- 2051 words;
 Dissertation_Roadmap_Meeting_20260727.docx</t>
+  </si>
+  <si>
+    <t>Refine the locator comprison map to make it clear to understand</t>
+  </si>
+  <si>
+    <t>No need to occupational analysis in the dissertation;
+Need to explicitly point out area names of case study in the results chapter for cascade mechanism comparison with class-3 gentrification subtypes</t>
+  </si>
+  <si>
+    <t>Refine locator map;
+Refine dissertation drafts and continue writing the remaining chapters</t>
+  </si>
+  <si>
+    <t>Dissertation roadmap for supervision meeting</t>
+  </si>
+  <si>
+    <t>flow_yee_palette.py;
+eda_12_v5_comparison_map_refined_20260729.ipynb;
+eda_10_v2_mechanism_case_locator_20260729.ipynb;
+results v6 - google drive --</t>
+  </si>
+  <si>
+    <t>flow_yee_palette.py;
+eda_12_v5_comparison_map_refined_20260729.ipynb;
+eda_10_v2_mechanism_case_locator_20260729.ipynb;
+eda_10_v3_mechanism_case_locator_20260729.ipynb
+results v6 - google drive</t>
   </si>
 </sst>
 </file>
@@ -3061,7 +3088,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4594,6 +4621,52 @@
       </c>
       <c r="H67" s="3" t="s">
         <v>254</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A68" s="2">
+        <v>46230</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H68" s="4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+      <c r="A69" s="2">
+        <v>46232</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added eda7 v3 - new alluvial plots - new colour palette and adding a new case for outflow-internal
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83B03036-4033-304D-9986-3FF98662BD32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB81CCB-7A6B-C540-BA1F-7AD8562ED999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2607,8 +2607,9 @@
   <si>
     <t>flow_yee_palette.py;
 eda_12_v5_comparison_map_refined_20260729.ipynb;
-eda_10_v2_mechanism_case_locator_20260729.ipynb;
-eda_10_v3_mechanism_case_locator_20260729.ipynb
+eda_10_v2 - v7_mechanism_case_locator_20260729.ipynb;
+eda_7_v3_case_decomposition_palette_and_westminster_20260729.ipynb;
+eda_5_v2_yee_flow_agreement_palette_20260729.ipynb
 results v6 - google drive</t>
   </si>
 </sst>

</xml_diff>

<commit_message>
Added eda12 v7 - new marker colour
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB81CCB-7A6B-C540-BA1F-7AD8562ED999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD84727-6837-DC4C-AFC6-1C22618DAF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2606,10 +2606,10 @@
   </si>
   <si>
     <t>flow_yee_palette.py;
-eda_12_v5_comparison_map_refined_20260729.ipynb;
+eda_12_v5-v7_comparison_map_refined_20260729.ipynb;
 eda_10_v2 - v7_mechanism_case_locator_20260729.ipynb;
 eda_7_v3_case_decomposition_palette_and_westminster_20260729.ipynb;
-eda_5_v2_yee_flow_agreement_palette_20260729.ipynb
+eda_5_v2&amp;v3_yee_flow_agreement_palette_20260729.ipynb
 results v6 - google drive</t>
   </si>
 </sst>

</xml_diff>

<commit_message>
Added eda3 rerun v2 - change new colour for each typology
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD84727-6837-DC4C-AFC6-1C22618DAF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F092A40D-D090-2047-BF93-0AFA9C1CD3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2609,7 +2609,8 @@
 eda_12_v5-v7_comparison_map_refined_20260729.ipynb;
 eda_10_v2 - v7_mechanism_case_locator_20260729.ipynb;
 eda_7_v3_case_decomposition_palette_and_westminster_20260729.ipynb;
-eda_5_v2&amp;v3_yee_flow_agreement_palette_20260729.ipynb
+eda_5_v2&amp;v3_yee_flow_agreement_palette_20260729.ipynb;
+eda_3_rerun_v2_typology_map_flow_yee_palette_20260729.ipynb
 results v6 - google drive</t>
   </si>
 </sst>
@@ -4650,7 +4651,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A69" s="2">
         <v>46232</v>
       </c>

</xml_diff>

<commit_message>
Added new versions of results and discussion chapter drafts
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F092A40D-D090-2047-BF93-0AFA9C1CD3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE1EE5F-EC8A-0A47-A9D8-84E0D9111E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="264">
   <si>
     <t>Date</t>
   </si>
@@ -2599,10 +2599,10 @@
     <t>Dissertation roadmap for supervision meeting</t>
   </si>
   <si>
-    <t>flow_yee_palette.py;
-eda_12_v5_comparison_map_refined_20260729.ipynb;
-eda_10_v2_mechanism_case_locator_20260729.ipynb;
-results v6 - google drive --</t>
+    <t>workflow pipeline diagram for methodology</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>flow_yee_palette.py;
@@ -2611,7 +2611,8 @@
 eda_7_v3_case_decomposition_palette_and_westminster_20260729.ipynb;
 eda_5_v2&amp;v3_yee_flow_agreement_palette_20260729.ipynb;
 eda_3_rerun_v2_typology_map_flow_yee_palette_20260729.ipynb
-results v6 - google drive</t>
+results v6 - google drive -- 2072 words;
+discussion v4 - google drive -- 2155 words</t>
   </si>
 </sst>
 </file>
@@ -3090,7 +3091,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4651,7 +4652,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A69" s="2">
         <v>46232</v>
       </c>
@@ -4659,16 +4660,27 @@
         <v>3</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>257</v>
       </c>
       <c r="E69" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="C73" s="3" t="s">
         <v>262</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added all version of workflow diagrams for methodology chapter draft - diagrams folder
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EE1EE5F-EC8A-0A47-A9D8-84E0D9111E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B838B3-8BF5-D14D-A63A-CA9C35BFB80D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="268">
   <si>
     <t>Date</t>
   </si>
@@ -2585,9 +2585,6 @@
 Dissertation_Roadmap_Meeting_20260727.docx</t>
   </si>
   <si>
-    <t>Refine the locator comprison map to make it clear to understand</t>
-  </si>
-  <si>
     <t>No need to occupational analysis in the dissertation;
 Need to explicitly point out area names of case study in the results chapter for cascade mechanism comparison with class-3 gentrification subtypes</t>
   </si>
@@ -2613,6 +2610,28 @@
 eda_3_rerun_v2_typology_map_flow_yee_palette_20260729.ipynb
 results v6 - google drive -- 2072 words;
 discussion v4 - google drive -- 2155 words</t>
+  </si>
+  <si>
+    <t>EDA;
+Dissertation draft</t>
+  </si>
+  <si>
+    <t>results v6 - google drive;
+discussion v4 - google drive;
+literature review v6 - google drive;
+methodology v15 - google drive</t>
+  </si>
+  <si>
+    <t>Refine the locator comparison map to make it clear to understand</t>
+  </si>
+  <si>
+    <t>Refine finished drafts;
+Create methodology workflow diagram(s)</t>
+  </si>
+  <si>
+    <t>literature review v6 - google drive;
+methodology v15 - google drive;
+workflow diagrams for methodology chapter</t>
   </si>
 </sst>
 </file>
@@ -4640,33 +4659,33 @@
         <v>23</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F68" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H68" s="4" t="s">
         <v>258</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H68" s="4" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="255" x14ac:dyDescent="0.2">
       <c r="A69" s="2">
         <v>46232</v>
       </c>
-      <c r="B69" s="3" t="s">
-        <v>3</v>
+      <c r="B69" s="4" t="s">
+        <v>263</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>23</v>
@@ -4675,12 +4694,29 @@
         <v>23</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>261</v>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A70" s="2">
+        <v>46233</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C73" s="3" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new verions of drafts - main changes in methodology
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65B838B3-8BF5-D14D-A63A-CA9C35BFB80D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DD01BC-729E-2249-9D31-B88304B39B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="269">
   <si>
     <t>Date</t>
   </si>
@@ -2616,12 +2616,6 @@
 Dissertation draft</t>
   </si>
   <si>
-    <t>results v6 - google drive;
-discussion v4 - google drive;
-literature review v6 - google drive;
-methodology v15 - google drive</t>
-  </si>
-  <si>
     <t>Refine the locator comparison map to make it clear to understand</t>
   </si>
   <si>
@@ -2632,6 +2626,15 @@
     <t>literature review v6 - google drive;
 methodology v15 - google drive;
 workflow diagrams for methodology chapter</t>
+  </si>
+  <si>
+    <t>results v6 - google drive -- 2072 words;
+discussion v4 - google drive -- 2107 words;
+literature review v6 - google drive -- 1826 words;
+methodology v15 - google drive -- 2907 words</t>
+  </si>
+  <si>
+    <t>appendix write-up</t>
   </si>
 </sst>
 </file>
@@ -3115,7 +3118,7 @@
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="38.83203125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="45.1640625" style="3" customWidth="1"/>
     <col min="4" max="4" width="75.1640625" style="3" customWidth="1"/>
     <col min="5" max="5" width="89.5" style="3" customWidth="1"/>
     <col min="6" max="6" width="151.33203125" style="3" customWidth="1"/>
@@ -4682,7 +4685,7 @@
         <v>262</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E69" s="4" t="s">
         <v>262</v>
@@ -4705,13 +4708,19 @@
         <v>239</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D70" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="E70" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="E70" s="4" t="s">
-        <v>267</v>
+      <c r="F70" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added appendix draft v0
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DD01BC-729E-2249-9D31-B88304B39B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE81DCB6-0138-B748-BBA4-4599D684F0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="274">
   <si>
     <t>Date</t>
   </si>
@@ -2635,6 +2635,27 @@
   </si>
   <si>
     <t>appendix write-up</t>
+  </si>
+  <si>
+    <t>Given details metioned in the methodology, how to draft the appendix efficiently?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the final version, there should be anything about the occupational ascent;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We do not need a sensitivity test for two different aggregation methods - modal-GEN/any-LSOA. Modal-GEN is used to construct a single categorical comparator; any-LSOA is used to detect the presence of overlapping subtype markers. Two methods are not overlapped with each other. Adding another sensivity test can blur the distiction between the aggregated GEN classification and the subtype indicators.
+</t>
+  </si>
+  <si>
+    <t>appendix v1 - google drive;
+methodology v16 - google drive - removed everything about occupational ascent &amp; explain any-LSOA/modal-GEN for Yee-label comparison;
+results v7 - google drive - clarify modal-GEN and any-LSOA</t>
+  </si>
+  <si>
+    <t>appendix v1 - google drive;
+methodology v16 - google drive -- 2971 words;
+results v7 - google drive -- 2093 words;</t>
   </si>
 </sst>
 </file>
@@ -4723,6 +4744,32 @@
         <v>268</v>
       </c>
     </row>
+    <row r="71" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A71" s="2">
+        <v>46234</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H71" s="4" t="s">
+        <v>270</v>
+      </c>
+    </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C73" s="3" t="s">
         <v>261</v>

</xml_diff>

<commit_message>
Updated appendix draft and small updates in according code files
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE81DCB6-0138-B748-BBA4-4599D684F0D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A639FC7-8B9D-AE42-8BDE-16B624BE8A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -2640,10 +2640,6 @@
     <t>Given details metioned in the methodology, how to draft the appendix efficiently?</t>
   </si>
   <si>
-    <t xml:space="preserve">In the final version, there should be anything about the occupational ascent;
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">We do not need a sensitivity test for two different aggregation methods - modal-GEN/any-LSOA. Modal-GEN is used to construct a single categorical comparator; any-LSOA is used to detect the presence of overlapping subtype markers. Two methods are not overlapped with each other. Adding another sensivity test can blur the distiction between the aggregated GEN classification and the subtype indicators.
 </t>
   </si>
@@ -2656,6 +2652,11 @@
     <t>appendix v1 - google drive;
 methodology v16 - google drive -- 2971 words;
 results v7 - google drive -- 2093 words;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Continue appendix write-up, from Appendix C.
+In the final version, there should be anything about the occupational ascent;
+</t>
   </si>
 </sst>
 </file>
@@ -4752,22 +4753,22 @@
         <v>239</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>269</v>
       </c>
       <c r="E71" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G71" s="3" t="s">
         <v>23</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated eda 7 - v4 - removed the kingston case from case 4
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A639FC7-8B9D-AE42-8BDE-16B624BE8A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4839F8-5E66-5345-80AE-670F24C62DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="278">
   <si>
     <t>Date</t>
   </si>
@@ -2657,6 +2657,27 @@
     <t xml:space="preserve">Continue appendix write-up, from Appendix C.
 In the final version, there should be anything about the occupational ascent;
 </t>
+  </si>
+  <si>
+    <t>Dissertation draft;
+EDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">redraw case study map, remove the kingston case
+</t>
+  </si>
+  <si>
+    <t>eda v1 rerun;
+results v8 - google drive;
+appendix v1 - google drive;
+eda 7 v4;
+eda 10 v8</t>
+  </si>
+  <si>
+    <t>eda v1 rerun (a cell output the correlation between cascade_dominance and CDS);
+results v8 - google drive;
+eda_7_v4_case_decomposition_palette_and_westminster_no_kingston_20260801.ipynb;
+eda_10_v8_mechanism_case_locator_no_kingston_20260801.ipynb</t>
   </si>
 </sst>
 </file>
@@ -4771,6 +4792,23 @@
         <v>273</v>
       </c>
     </row>
+    <row r="72" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A72" s="2">
+        <v>46235</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>275</v>
+      </c>
+    </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="C73" s="3" t="s">
         <v>261</v>

</xml_diff>

<commit_message>
Finished appendix draft v1
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4839F8-5E66-5345-80AE-670F24C62DB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0F70F8-4E8D-8C4E-AA6B-9065ADEF41FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="278">
   <si>
     <t>Date</t>
   </si>
@@ -2663,10 +2663,6 @@
 EDA</t>
   </si>
   <si>
-    <t xml:space="preserve">redraw case study map, remove the kingston case
-</t>
-  </si>
-  <si>
     <t>eda v1 rerun;
 results v8 - google drive;
 appendix v1 - google drive;
@@ -2678,6 +2674,10 @@
 results v8 - google drive;
 eda_7_v4_case_decomposition_palette_and_westminster_no_kingston_20260801.ipynb;
 eda_10_v8_mechanism_case_locator_no_kingston_20260801.ipynb</t>
+  </si>
+  <si>
+    <t>After the full read across chapters, need to consider the weights between each chapter. Methodology may need more from current appendices.;
+Start to write conclusion and introduction.</t>
   </si>
 </sst>
 </file>
@@ -4800,13 +4800,22 @@
         <v>274</v>
       </c>
       <c r="C72" s="4" t="s">
+        <v>275</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="E72" s="4" t="s">
+      <c r="F72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H72" s="4" t="s">
         <v>277</v>
-      </c>
-      <c r="H72" s="4" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Finished appendices draft v2 - added other refined chapter drafts
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0F70F8-4E8D-8C4E-AA6B-9065ADEF41FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E9553C2-C04D-6042-984F-0083C18575AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="281">
   <si>
     <t>Date</t>
   </si>
@@ -2599,9 +2599,6 @@
     <t>workflow pipeline diagram for methodology</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>flow_yee_palette.py;
 eda_12_v5-v7_comparison_map_refined_20260729.ipynb;
 eda_10_v2 - v7_mechanism_case_locator_20260729.ipynb;
@@ -2678,6 +2675,24 @@
   <si>
     <t>After the full read across chapters, need to consider the weights between each chapter. Methodology may need more from current appendices.;
 Start to write conclusion and introduction.</t>
+  </si>
+  <si>
+    <t>Literature review and appendix revise - after the full read - follow advice</t>
+  </si>
+  <si>
+    <t>methodology v17 --- 2812 words;
+appendix v2;
+results v9 --  2007 words;
+discussion v5 -- 1884 words</t>
+  </si>
+  <si>
+    <t>According to drafted appendices, refine the rest of drafts if they're cimbined as a full paper.</t>
+  </si>
+  <si>
+    <t>methodology v17;
+appendix v2;
+results v9;
+discussion v5</t>
   </si>
 </sst>
 </file>
@@ -4722,16 +4737,16 @@
         <v>46232</v>
       </c>
       <c r="B69" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="D69" s="3" t="s">
         <v>263</v>
       </c>
-      <c r="C69" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>264</v>
-      </c>
       <c r="E69" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F69" s="3" t="s">
         <v>23</v>
@@ -4751,19 +4766,19 @@
         <v>239</v>
       </c>
       <c r="C70" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H70" s="3" t="s">
         <v>267</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="E70" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="F70" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H70" s="3" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -4774,22 +4789,22 @@
         <v>239</v>
       </c>
       <c r="C71" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H71" s="4" t="s">
         <v>272</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="F71" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H71" s="4" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="85" x14ac:dyDescent="0.2">
@@ -4797,30 +4812,51 @@
         <v>46235</v>
       </c>
       <c r="B72" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="C72" s="4" t="s">
         <v>274</v>
       </c>
-      <c r="C72" s="4" t="s">
+      <c r="D72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="D72" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E72" s="4" t="s">
+      <c r="F72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H72" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="F72" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G72" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H72" s="4" t="s">
+    </row>
+    <row r="73" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A73" s="2">
+        <v>46236</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H73" s="3" t="s">
         <v>277</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C73" s="3" t="s">
-        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new versions of analytical pipeline diagrams
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E9553C2-C04D-6042-984F-0083C18575AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BCBCEA1-B487-AE45-8C4C-EE51088310D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="283">
   <si>
     <t>Date</t>
   </si>
@@ -2693,6 +2693,14 @@
 appendix v2;
 results v9;
 discussion v5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">literature review v7 --- ;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">literature review v7;
+</t>
   </si>
 </sst>
 </file>
@@ -3171,7 +3179,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H73"/>
+  <dimension ref="A1:H74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4857,6 +4865,20 @@
       </c>
       <c r="H73" s="3" t="s">
         <v>277</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A74" s="2">
+        <v>46237</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added integrated drafts - partly
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BCBCEA1-B487-AE45-8C4C-EE51088310D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA8FC07-EB58-1445-9E5E-BF240D0B6E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="289">
   <si>
     <t>Date</t>
   </si>
@@ -2695,12 +2695,41 @@
 discussion v5</t>
   </si>
   <si>
-    <t xml:space="preserve">literature review v7 --- ;
+    <t>literature review v7 --- 1834 words;
+methodology v18 --- 2852 words</t>
+  </si>
+  <si>
+    <t>literature review v7;
+methodology v18</t>
+  </si>
+  <si>
+    <t>Check the overlap in appendices among other chapters;
+Based on new RQs and the structure, refine the resuls and discussion chapters.</t>
+  </si>
+  <si>
+    <t>results v10;
+discussion v6;
+partly-integrated-draft</t>
+  </si>
+  <si>
+    <t>RQs refined: To what extent do hierarchy-crossing migration structures correspond with independently identified neighbourhood ascent and gentrification subtypes? (Correspondence)
+How general is the proposed cascade structure across census periods and alternative deprivation and geographical reference frames? (Generality) 
+Which combinations of inflow and outflow underlie the coarse cascade classification, and how do they correspond with specific gentrification subtypes? (Mechanism)</t>
+  </si>
+  <si>
+    <t>How to make each chapter logically connected without any overlaps?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">results v10;
+discussion v6;
+partly-integrated-draft;
+partly-integrated-draft-v2-20260804
 </t>
   </si>
   <si>
-    <t xml:space="preserve">literature review v7;
-</t>
+    <t>Check the full integrated drafts - summarise each subsection to see the logic of the whole story and the connection;
+Check repititions;
+Start to write intro and conclusion</t>
   </si>
 </sst>
 </file>
@@ -3179,7 +3208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -4867,7 +4896,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A74" s="2">
         <v>46237</v>
       </c>
@@ -4877,8 +4906,46 @@
       <c r="C74" s="4" t="s">
         <v>281</v>
       </c>
+      <c r="D74" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="E74" s="4" t="s">
         <v>282</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H74" s="4" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A75" s="2">
+        <v>46238</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G75" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H75" s="4" t="s">
+        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the integrated draft - v3
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA8FC07-EB58-1445-9E5E-BF240D0B6E64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4F87FA-14C1-9D45-ADD5-422FFA59F1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="292">
   <si>
     <t>Date</t>
   </si>
@@ -2730,6 +2730,17 @@
     <t>Check the full integrated drafts - summarise each subsection to see the logic of the whole story and the connection;
 Check repititions;
 Start to write intro and conclusion</t>
+  </si>
+  <si>
+    <t>partly-integrated-draft-v3-20260805</t>
+  </si>
+  <si>
+    <t>Make the RQs not post-hoc;
+Check across chapters and sections to avoid repetitions and make the logic well connected</t>
+  </si>
+  <si>
+    <t>Intro and conclusion write-up;
+Full read by sentence.</t>
   </si>
 </sst>
 </file>
@@ -2851,16 +2862,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2869,10 +2871,19 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3208,7 +3219,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -3457,70 +3468,70 @@
       </c>
     </row>
     <row r="12" spans="1:8" s="5" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="F12" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" s="10" t="s">
+      <c r="G12" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H12" s="8" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="15"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
+      <c r="A13" s="13"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="8" t="s">
+      <c r="D14" s="12"/>
+      <c r="E14" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="14"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="8" t="s">
+      <c r="F14" s="12"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="11" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="13"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="8"/>
+      <c r="A15" s="10"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="11"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
@@ -3544,43 +3555,43 @@
       <c r="G16" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H16" s="8" t="s">
+      <c r="H16" s="11" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="D17" s="8" t="s">
+      <c r="D17" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="H17" s="8"/>
+      <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="13"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
+      <c r="A18" s="10"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
@@ -3612,25 +3623,25 @@
       <c r="A20" s="2">
         <v>46178</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="B20" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D20" s="9" t="s">
+      <c r="C20" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D20" s="14" t="s">
         <v>87</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="F20" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H20" s="8" t="s">
+      <c r="F20" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="H20" s="11" t="s">
         <v>23</v>
       </c>
     </row>
@@ -3638,43 +3649,43 @@
       <c r="A21" s="2">
         <v>46179</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="14"/>
       <c r="E21" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="11"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>46180</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="14"/>
       <c r="E22" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>46181</v>
       </c>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="14"/>
       <c r="E23" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11"/>
+      <c r="H23" s="11"/>
     </row>
     <row r="24" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
@@ -3706,7 +3717,7 @@
       <c r="A25" s="2">
         <v>46183</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="11" t="s">
         <v>93</v>
       </c>
       <c r="C25" s="4" t="s">
@@ -3724,7 +3735,7 @@
       <c r="G25" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="14" t="s">
         <v>97</v>
       </c>
     </row>
@@ -3732,7 +3743,7 @@
       <c r="A26" s="2">
         <v>46184</v>
       </c>
-      <c r="B26" s="8"/>
+      <c r="B26" s="11"/>
       <c r="C26" s="4" t="s">
         <v>95</v>
       </c>
@@ -3748,13 +3759,13 @@
       <c r="G26" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="H26" s="9"/>
+      <c r="H26" s="14"/>
     </row>
     <row r="27" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>46185</v>
       </c>
-      <c r="B27" s="8"/>
+      <c r="B27" s="11"/>
       <c r="C27" s="4" t="s">
         <v>101</v>
       </c>
@@ -3770,13 +3781,13 @@
       <c r="G27" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="H27" s="9"/>
+      <c r="H27" s="14"/>
     </row>
     <row r="28" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>46186</v>
       </c>
-      <c r="B28" s="8"/>
+      <c r="B28" s="11"/>
       <c r="C28" s="4" t="s">
         <v>104</v>
       </c>
@@ -3792,13 +3803,13 @@
       <c r="G28" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="H28" s="9"/>
+      <c r="H28" s="14"/>
     </row>
     <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>46187</v>
       </c>
-      <c r="B29" s="8"/>
+      <c r="B29" s="11"/>
       <c r="C29" s="4" t="s">
         <v>107</v>
       </c>
@@ -3822,7 +3833,7 @@
       <c r="A30" s="2">
         <v>46188</v>
       </c>
-      <c r="B30" s="8"/>
+      <c r="B30" s="11"/>
       <c r="C30" s="4" t="s">
         <v>113</v>
       </c>
@@ -3838,7 +3849,7 @@
       <c r="G30" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H30" s="8" t="s">
+      <c r="H30" s="11" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3846,61 +3857,61 @@
       <c r="A31" s="2">
         <v>46189</v>
       </c>
-      <c r="B31" s="8" t="s">
+      <c r="B31" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="11" t="s">
         <v>119</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="F31" s="9" t="s">
+      <c r="F31" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="H31" s="8"/>
+      <c r="H31" s="11"/>
     </row>
     <row r="32" spans="1:8" ht="92" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>46190</v>
       </c>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
       <c r="D32" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E32" s="8"/>
-      <c r="F32" s="9"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
     </row>
     <row r="33" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>46191</v>
       </c>
-      <c r="B33" s="8"/>
-      <c r="C33" s="9" t="s">
+      <c r="B33" s="11"/>
+      <c r="C33" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G33" s="9" t="s">
+      <c r="G33" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="H33" s="9" t="s">
+      <c r="H33" s="14" t="s">
         <v>9</v>
       </c>
     </row>
@@ -3908,19 +3919,19 @@
       <c r="A34" s="2">
         <v>46192</v>
       </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="9"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
+      <c r="B34" s="11"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
     </row>
     <row r="35" spans="1:8" ht="268" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>46193</v>
       </c>
-      <c r="B35" s="8"/>
+      <c r="B35" s="11"/>
       <c r="C35" s="4" t="s">
         <v>124</v>
       </c>
@@ -4167,7 +4178,7 @@
       <c r="G44" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="H44" s="10" t="s">
+      <c r="H44" s="8" t="s">
         <v>180</v>
       </c>
     </row>
@@ -4181,7 +4192,7 @@
       <c r="C45" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" s="8" t="s">
         <v>182</v>
       </c>
       <c r="E45" s="3" t="s">
@@ -4190,10 +4201,10 @@
       <c r="F45" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G45" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="H45" s="10"/>
+      <c r="G45" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H45" s="8"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
@@ -4205,15 +4216,15 @@
       <c r="C46" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D46" s="10"/>
+      <c r="D46" s="8"/>
       <c r="E46" s="3" t="s">
         <v>184</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G46" s="10"/>
-      <c r="H46" s="10"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="8"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
@@ -4225,15 +4236,15 @@
       <c r="C47" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D47" s="10"/>
+      <c r="D47" s="8"/>
       <c r="E47" s="3" t="s">
         <v>185</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
+      <c r="G47" s="8"/>
+      <c r="H47" s="8"/>
     </row>
     <row r="48" spans="1:8" ht="204" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
@@ -4245,15 +4256,15 @@
       <c r="C48" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D48" s="10"/>
+      <c r="D48" s="8"/>
       <c r="E48" s="3" t="s">
         <v>186</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
     </row>
     <row r="49" spans="1:8" ht="136" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
@@ -4948,20 +4959,48 @@
         <v>288</v>
       </c>
     </row>
+    <row r="76" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A76" s="2">
+        <v>46239</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>291</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D12:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F12:F15"/>
-    <mergeCell ref="G12:G15"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="D45:D48"/>
+    <mergeCell ref="G45:G48"/>
+    <mergeCell ref="H44:H48"/>
+    <mergeCell ref="C33:C34"/>
+    <mergeCell ref="D33:D34"/>
+    <mergeCell ref="H33:H34"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="F33:F34"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="B25:B30"/>
+    <mergeCell ref="H25:H28"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H30:H32"/>
     <mergeCell ref="H20:H23"/>
     <mergeCell ref="H14:H15"/>
     <mergeCell ref="A17:A18"/>
@@ -4977,23 +5016,18 @@
     <mergeCell ref="D20:D23"/>
     <mergeCell ref="F20:F23"/>
     <mergeCell ref="G20:G23"/>
-    <mergeCell ref="B25:B30"/>
-    <mergeCell ref="H25:H28"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="D45:D48"/>
-    <mergeCell ref="G45:G48"/>
-    <mergeCell ref="H44:H48"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="H30:H32"/>
-    <mergeCell ref="H33:H34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F12:F15"/>
+    <mergeCell ref="G12:G15"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="E12:E13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finished the final complete version
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{031D57F1-14A5-0243-A5CD-AE0732F8BC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100A590F-9292-A546-A53C-D18DC0159B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="304">
   <si>
     <t>Date</t>
   </si>
@@ -2771,6 +2771,16 @@
   <si>
     <t>Preamble, abstract, research log, acknowledgement, bibliography;
 GitHub orgainsing</t>
+  </si>
+  <si>
+    <t>Front pages</t>
+  </si>
+  <si>
+    <t>partly-integrated-draft-v4-20260807;
+integrated-draft-v5-20260809</t>
+  </si>
+  <si>
+    <t>Email Adam with final version for submission check.</t>
   </si>
 </sst>
 </file>
@@ -3249,7 +3259,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
@@ -5065,6 +5075,32 @@
       </c>
       <c r="H78" s="4" t="s">
         <v>300</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A79" s="2">
+        <v>46243</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="E79" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="F79" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update README; Updated research logbook
</commit_message>
<xml_diff>
--- a/research-logbook.xlsx
+++ b/research-logbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xing/Desktop/CASA/dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{100A590F-9292-A546-A53C-D18DC0159B67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4906FE24-8381-C745-A433-F893417EB347}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5820" yWindow="660" windowWidth="24420" windowHeight="17860" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17320" xr2:uid="{1EE6576A-BED4-1C49-93D2-9A0D58957AE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="340">
   <si>
     <t>Date</t>
   </si>
@@ -146,22 +146,7 @@
     <t>Email Adam with latest drafts for review.</t>
   </si>
   <si>
-    <t>How to structure the methodology draft structure? 
-(Writing the dissertation)</t>
-  </si>
-  <si>
     <t>Draft in methodology (Google file) v7</t>
-  </si>
-  <si>
-    <t>Methodology pipeline diagram</t>
-  </si>
-  <si>
-    <t>More literature reviews on terminology.</t>
-  </si>
-  <si>
-    <t>How to explain terminology in a more accurate and logic way and connect them coherently?
-Need deeper understanding in terminology (e.g. deprivation gradient, deprivation hierarchy, displacement pressure, etc.).
-(See detailed comments in the draft)</t>
   </si>
   <si>
     <t>methodology (Google file);
@@ -170,9 +155,6 @@
   <si>
     <t>Methodology;
 Conceptual Framework</t>
-  </si>
-  <si>
-    <t>Draft in Methodology(Google file) v1 &amp; v2</t>
   </si>
   <si>
     <t>Draft in Methodology(Google file) v4</t>
@@ -753,9 +735,6 @@
   <si>
     <t>Data preprocess;
 EDA</t>
-  </si>
-  <si>
-    <t>data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb</t>
   </si>
   <si>
     <t xml:space="preserve">data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb;
@@ -2781,6 +2760,168 @@
   </si>
   <si>
     <t>Email Adam with final version for submission check.</t>
+  </si>
+  <si>
+    <t>Literature review;
+Code organisation</t>
+  </si>
+  <si>
+    <t>Aspect_of_change-reading_notes - reading archive</t>
+  </si>
+  <si>
+    <t>(updated)Aspect_of_change-reading_notes</t>
+  </si>
+  <si>
+    <t>(updated)Aspect_of_change-reading_notes;
+New main branch of the repo - cleaned and organised code files and descriptions</t>
+  </si>
+  <si>
+    <t>(updated)Aspect_of_change-reading_notes;
+Check and run all cleaned code files and outputs</t>
+  </si>
+  <si>
+    <t>Research proposal</t>
+  </si>
+  <si>
+    <t>What can I do for this dissertation;
+Which topic should I work on</t>
+  </si>
+  <si>
+    <t>From papers about LCR, it's quite interesting to explore flows under the topic of gentrification, most studies used attribute-based indicators to discuss the consequences of gentrification</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>Can we use a flow-based method to discuss gentrification?</t>
+  </si>
+  <si>
+    <t>More detailed proposal idea;
+Supervision match</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>Given the Census OD data, what are the basic/initial findings in London, in terms of gentrification?
+What’s the next direction to explore?</t>
+  </si>
+  <si>
+    <t>Given we have 2 census periods, we should decide the design of deprivation hierarchy, if we want to explore the migration as hierarchy-crossing movements.
+All cascade metrics show high correlation (r &gt; 0.82) between the 2010 and 2019 baseline classifications, for both the 2011 and 2021 OD data.
+The sign and significance of correlations between cascade metrics and IMD Percentile Change are consistent across baselines.
+CFI Rate at the borough level shows concordance of r ≈ 0.89 (CFI Rate) and 0.99 (CFI Churn) between baselines, and validation correlations with IMD Percentile Change remain consistent.</t>
+  </si>
+  <si>
+    <t>How to decide the reference frame choice?</t>
+  </si>
+  <si>
+    <t>Supervision meeting</t>
+  </si>
+  <si>
+    <t>(Meeting with Adam)
+data_preprocess_add_outerLondon_as_another_MSOA_20260622.ipynb</t>
+  </si>
+  <si>
+    <t>How to refine the analysis methodology for cascading?</t>
+  </si>
+  <si>
+    <t>More EDA;
+data preprocessing with 2011 OD data</t>
+  </si>
+  <si>
+    <t>Need to be care about the analysis method with IMD - shouldn't use IMD raw scores to compare;
+We need 2011 OD data</t>
+  </si>
+  <si>
+    <t>eda_adding_2011oddata</t>
+  </si>
+  <si>
+    <t>How to extend analysis with both 2011 and 2021 OD data</t>
+  </si>
+  <si>
+    <t>(see interpretation in the eda file)</t>
+  </si>
+  <si>
+    <t>How to get all data we need to use?</t>
+  </si>
+  <si>
+    <t>Extension on 2011 OD data</t>
+  </si>
+  <si>
+    <t>EDA;
+Literature review;
+Dissertation draft</t>
+  </si>
+  <si>
+    <t>eda_update_cascade_features;
+methodology - google drive</t>
+  </si>
+  <si>
+    <t>How to design cascade features for further analysis</t>
+  </si>
+  <si>
+    <t>Cascade feature design</t>
+  </si>
+  <si>
+    <t>Data preprocess;
+Literature review</t>
+  </si>
+  <si>
+    <t>eda-v1;
+eda-v1.5</t>
+  </si>
+  <si>
+    <t>data_process_update_imd_rank_analysis;
+eda_cascade_analysis_imd_score;
+eda_cascade_bivariate_analysis;
+eda_cascade_imd_rank_analysis;
+eda-v2-meeting</t>
+  </si>
+  <si>
+    <t>How to analyse IMD with rank?</t>
+  </si>
+  <si>
+    <t>data_process_update_imd_rank_analysis;
+eda_cascade_analysis_imd_score;
+eda_cascade_bivariate_analysis;
+eda_cascade_imd_rank_analysis;
+eda-v2-meeting;
+all eda outputs</t>
+  </si>
+  <si>
+    <t>How to understand the relationship between cascade and IMD change?</t>
+  </si>
+  <si>
+    <t>Create some interactive visualisation to show the flows</t>
+  </si>
+  <si>
+    <t>How to make flow interactive visualisations?</t>
+  </si>
+  <si>
+    <t>Nomis has their own interactive visualisation for OD only for 2021 migration.</t>
+  </si>
+  <si>
+    <t>Could these visualisation show what we want in the dissertation?
+Or maybe there could be a better refinement for visualisation?</t>
+  </si>
+  <si>
+    <t>Data visualisation;
+EDA;
+Data preprocess;
+Literature review</t>
+  </si>
+  <si>
+    <t>butterfly_chart.py;
+cascade_explorer.py &amp; .html;
+cascade_combined_flow.jsx;
+eda_cascade_imd_rank_analysis;
+data_process_prepare_2019baseline;
+eda_adding_2011oddata</t>
+  </si>
+  <si>
+    <t>workflow pipeline diagram;
+Keep writing up the methodology and organising the conceptual framework</t>
   </si>
 </sst>
 </file>
@@ -2904,6 +3045,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2911,19 +3061,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3259,11 +3400,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18C40938-6431-324A-A7B6-6768F21B6E05}">
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.83203125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="45.1640625" style="3" customWidth="1"/>
     <col min="4" max="4" width="75.1640625" style="3" customWidth="1"/>
     <col min="5" max="5" width="89.5" style="3" customWidth="1"/>
@@ -3299,1308 +3440,1363 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>45796</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>27</v>
+        <v>46125</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>68</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>28</v>
+        <v>89</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>33</v>
+        <v>310</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>45797</v>
+        <v>46151</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>35</v>
+        <v>135</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>318</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>41</v>
+        <v>319</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>318</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>44</v>
+        <v>320</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>45798</v>
+        <v>46154</v>
       </c>
       <c r="B6" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>46157</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="119" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>46160</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
+        <v>46163</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="H11" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C6" s="4" t="s">
+    </row>
+    <row r="12" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D12" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>46165</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" s="4" t="s">
+      <c r="C13" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
-        <v>45799</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="4" t="s">
+      <c r="H13" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
+        <v>46166</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A8" s="2">
-        <v>45800</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="C14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="G14" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A9" s="2">
-        <v>45801</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" s="4" t="s">
+    </row>
+    <row r="15" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>46167</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E15" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="221" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>46168</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A10" s="2">
-        <v>45802</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="221" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
-        <v>46168</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="5" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="13" t="s">
+    <row r="17" spans="1:8" s="5" customFormat="1" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="15" t="s">
         <v>25</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A14" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="11"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="2">
-        <v>46174</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A17" s="9" t="s">
-        <v>76</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="H17" s="11"/>
-    </row>
-    <row r="18" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10"/>
+      <c r="C17" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A18" s="15"/>
       <c r="B18" s="8"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-    </row>
-    <row r="19" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A19" s="2">
-        <v>46177</v>
-      </c>
-      <c r="B19" s="3" t="s">
+      <c r="C18" s="8"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="2">
-        <v>46178</v>
-      </c>
-      <c r="B20" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H20" s="11" t="s">
-        <v>23</v>
-      </c>
+      <c r="D19" s="14"/>
+      <c r="E19" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F19" s="14"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" s="13"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="10"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
+        <v>46174</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A22" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G22" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="H22" s="10"/>
+    </row>
+    <row r="23" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="13"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+    </row>
+    <row r="24" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>46177</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
+        <v>46178</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" s="2">
         <v>46179</v>
       </c>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="F21" s="11"/>
-      <c r="G21" s="11"/>
-      <c r="H21" s="11"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A22" s="2">
+      <c r="B26" s="10"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F26" s="10"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="10"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A27" s="2">
         <v>46180</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A23" s="2">
+      <c r="B27" s="10"/>
+      <c r="C27" s="10"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F27" s="10"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A28" s="2">
         <v>46181</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
-    </row>
-    <row r="24" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A24" s="2">
-        <v>46182</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A25" s="2">
-        <v>46183</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A26" s="2">
-        <v>46184</v>
-      </c>
-      <c r="B26" s="11"/>
-      <c r="C26" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="H26" s="14"/>
-    </row>
-    <row r="27" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A27" s="2">
-        <v>46185</v>
-      </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="H27" s="14"/>
-    </row>
-    <row r="28" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A28" s="2">
-        <v>46186</v>
-      </c>
-      <c r="B28" s="11"/>
-      <c r="C28" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D28" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="F28" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="H28" s="14"/>
+      <c r="B28" s="10"/>
+      <c r="C28" s="10"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="F28" s="10"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
     </row>
     <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
-        <v>46187</v>
-      </c>
-      <c r="B29" s="11"/>
-      <c r="C29" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="F29" s="4" t="s">
-        <v>111</v>
+        <v>46182</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>110</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
+        <v>46183</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A31" s="2">
+        <v>46184</v>
+      </c>
+      <c r="B31" s="10"/>
+      <c r="C31" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="H31" s="9"/>
+    </row>
+    <row r="32" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A32" s="2">
+        <v>46185</v>
+      </c>
+      <c r="B32" s="10"/>
+      <c r="C32" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H32" s="9"/>
+    </row>
+    <row r="33" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>46186</v>
+      </c>
+      <c r="B33" s="10"/>
+      <c r="C33" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="H33" s="9"/>
+    </row>
+    <row r="34" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A34" s="2">
+        <v>46187</v>
+      </c>
+      <c r="B34" s="10"/>
+      <c r="C34" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
         <v>46188</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="4" t="s">
+      <c r="B35" s="10"/>
+      <c r="C35" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>46189</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G36" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="H36" s="10"/>
+    </row>
+    <row r="37" spans="1:8" ht="92" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>46190</v>
+      </c>
+      <c r="B37" s="10"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G30" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H30" s="11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="2">
-        <v>46189</v>
-      </c>
-      <c r="B31" s="11" t="s">
+      <c r="E37" s="10"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="10"/>
+    </row>
+    <row r="38" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="2">
+        <v>46191</v>
+      </c>
+      <c r="B38" s="10"/>
+      <c r="C38" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H38" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="2">
+        <v>46192</v>
+      </c>
+      <c r="B39" s="10"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+    </row>
+    <row r="40" spans="1:8" ht="268" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="2">
+        <v>46193</v>
+      </c>
+      <c r="B40" s="10"/>
+      <c r="C40" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="409" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="2">
+        <v>46194</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="170" x14ac:dyDescent="0.2">
+      <c r="A42" s="2">
+        <v>46195</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="G42" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="221" x14ac:dyDescent="0.2">
+      <c r="A43" s="2">
+        <v>46196</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A44" s="2">
+        <v>46197</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E44" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="G44" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="272" x14ac:dyDescent="0.2">
+      <c r="A45" s="2">
+        <v>46198</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="409.5" x14ac:dyDescent="0.2">
+      <c r="A46" s="2">
+        <v>46199</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G46" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
+        <v>46200</v>
+      </c>
+      <c r="B47" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C31" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="F31" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="G31" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="H31" s="11"/>
-    </row>
-    <row r="32" spans="1:8" ht="92" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="2">
-        <v>46190</v>
-      </c>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="E32" s="11"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-    </row>
-    <row r="33" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="2">
-        <v>46191</v>
-      </c>
-      <c r="B33" s="11"/>
-      <c r="C33" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H33" s="14" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="2">
-        <v>46192</v>
-      </c>
-      <c r="B34" s="11"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-    </row>
-    <row r="35" spans="1:8" ht="268" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="2">
-        <v>46193</v>
-      </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="H35" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="409" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="2">
-        <v>46194</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="170" x14ac:dyDescent="0.2">
-      <c r="A37" s="2">
-        <v>46195</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="D37" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="F37" s="4" t="s">
+      <c r="C47" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="306" x14ac:dyDescent="0.2">
+      <c r="A48" s="2">
+        <v>46201</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A49" s="2">
+        <v>46202</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D49" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="G37" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="H37" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="221" x14ac:dyDescent="0.2">
-      <c r="A38" s="2">
-        <v>46196</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="D38" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="F38" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="H38" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A39" s="2">
-        <v>46197</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="272" x14ac:dyDescent="0.2">
-      <c r="A40" s="2">
-        <v>46198</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="F40" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="409.5" x14ac:dyDescent="0.2">
-      <c r="A41" s="2">
-        <v>46199</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="204" x14ac:dyDescent="0.2">
-      <c r="A42" s="2">
-        <v>46200</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="G42" s="4" t="s">
+      <c r="E49" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="H49" s="8" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="2">
+        <v>46203</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="H42" s="4" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="306" x14ac:dyDescent="0.2">
-      <c r="A43" s="2">
-        <v>46201</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="D43" s="4" t="s">
+      <c r="F50" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G50" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H50" s="8"/>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="2">
+        <v>46204</v>
+      </c>
+      <c r="B51" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C51" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="E43" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A44" s="2">
-        <v>46202</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D44" s="3" t="s">
+      <c r="D51" s="8"/>
+      <c r="E51" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="E44" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F44" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G44" s="4" t="s">
+      <c r="F51" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G51" s="8"/>
+      <c r="H51" s="8"/>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="2">
+        <v>46205</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D52" s="8"/>
+      <c r="E52" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="H44" s="8" t="s">
+      <c r="F52" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8"/>
+    </row>
+    <row r="53" spans="1:8" ht="204" x14ac:dyDescent="0.2">
+      <c r="A53" s="2">
+        <v>46206</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D53" s="8"/>
+      <c r="E53" s="3" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A45" s="2">
-        <v>46203</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C45" s="3" t="s">
+      <c r="F53" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+    </row>
+    <row r="54" spans="1:8" ht="136" x14ac:dyDescent="0.2">
+      <c r="A54" s="2">
+        <v>46207</v>
+      </c>
+      <c r="B54" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="E45" s="3" t="s">
+      <c r="C54" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E54" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="F45" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G45" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H45" s="8"/>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A46" s="2">
-        <v>46204</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D46" s="8"/>
-      <c r="E46" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="F46" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A47" s="2">
-        <v>46205</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D47" s="8"/>
-      <c r="E47" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
-    </row>
-    <row r="48" spans="1:8" ht="204" x14ac:dyDescent="0.2">
-      <c r="A48" s="2">
-        <v>46206</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="D48" s="8"/>
-      <c r="E48" s="3" t="s">
+      <c r="F54" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G54" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="H54" s="4" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="187" x14ac:dyDescent="0.2">
+      <c r="A55" s="2">
+        <v>46208</v>
+      </c>
+      <c r="B55" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="G48" s="8"/>
-      <c r="H48" s="8"/>
-    </row>
-    <row r="49" spans="1:8" ht="136" x14ac:dyDescent="0.2">
-      <c r="A49" s="2">
-        <v>46207</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="C49" s="4" t="s">
+      <c r="C55" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="D55" s="4" t="s">
         <v>190</v>
       </c>
-      <c r="D49" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="F49" s="4" t="s">
+      <c r="E55" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="G49" s="4" t="s">
+      <c r="F55" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="G55" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="H49" s="4" t="s">
+      <c r="H55" s="4" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="187" x14ac:dyDescent="0.2">
-      <c r="A50" s="2">
-        <v>46208</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C50" s="4" t="s">
+    <row r="56" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A56" s="2">
+        <v>46209</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="D56" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="D50" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="E50" s="4" t="s">
+      <c r="E56" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A57" s="2">
+        <v>46211</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D57" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="F50" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>198</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A51" s="2">
-        <v>46209</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="D51" s="3" t="s">
+      <c r="E57" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="E51" s="4" t="s">
+      <c r="F57" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="F51" s="3" t="s">
+      <c r="G57" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A58" s="2">
+        <v>46212</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="G51" s="4" t="s">
+      <c r="D58" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="H51" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A52" s="2">
-        <v>46211</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C52" s="4" t="s">
+      <c r="E58" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H58" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="D52" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="E52" s="4" t="s">
+    </row>
+    <row r="59" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A59" s="2">
+        <v>46214</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E59" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="F52" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A53" s="2">
-        <v>46212</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="F53" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G53" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H53" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A54" s="2">
-        <v>46214</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="F54" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H54" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A55" s="2">
-        <v>46215</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G55" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H55" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A56" s="2">
-        <v>46216</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="F56" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A57" s="2">
-        <v>46217</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="D57" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E57" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="H57" s="3" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A58" s="2">
-        <v>46218</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="E58" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="H58" s="3" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" ht="119" x14ac:dyDescent="0.2">
-      <c r="A59" s="2">
-        <v>46219</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="D59" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="E59" s="4" t="s">
-        <v>234</v>
-      </c>
       <c r="F59" s="3" t="s">
         <v>23</v>
       </c>
       <c r="G59" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H59" s="6" t="s">
-        <v>233</v>
+      <c r="H59" s="3" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
-        <v>46221</v>
+        <v>46215</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>239</v>
+        <v>68</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>23</v>
+        <v>206</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>235</v>
+        <v>23</v>
       </c>
       <c r="F60" s="3" t="s">
         <v>23</v>
@@ -4609,546 +4805,768 @@
         <v>23</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>237</v>
+        <v>208</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
-        <v>46222</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>239</v>
+        <v>46216</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>210</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>241</v>
+        <v>205</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>206</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="F61" s="3" t="s">
-        <v>236</v>
+        <v>23</v>
       </c>
       <c r="G61" s="3" t="s">
         <v>23</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
-        <v>46223</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>242</v>
+        <v>46217</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>216</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>243</v>
+        <v>215</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>214</v>
       </c>
       <c r="F62" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>23</v>
+        <v>217</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>218</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
-        <v>46224</v>
+        <v>46218</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G63" s="3" t="s">
-        <v>23</v>
+        <v>3</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>223</v>
       </c>
       <c r="H63" s="3" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="119" x14ac:dyDescent="0.2">
       <c r="A64" s="2">
-        <v>46226</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>251</v>
+        <v>46219</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>225</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>247</v>
+        <v>226</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="F64" s="4" t="s">
-        <v>245</v>
+        <v>228</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>23</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="H64" s="3" t="s">
-        <v>244</v>
+      <c r="H64" s="6" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="2">
+        <v>46221</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A66" s="2">
+        <v>46222</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A67" s="2">
+        <v>46223</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A68" s="2">
+        <v>46224</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A69" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A70" s="2">
         <v>46227</v>
       </c>
-      <c r="B65" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C65" s="3" t="s">
+      <c r="B70" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A71" s="2">
+        <v>46228</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+      <c r="A72" s="2">
+        <v>46229</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D65" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E65" s="3" t="s">
+      <c r="F72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H72" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="F65" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H65" s="3" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A66" s="2">
-        <v>46228</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C66" s="4" t="s">
+    </row>
+    <row r="73" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A73" s="2">
+        <v>46230</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H73" s="4" t="s">
         <v>252</v>
       </c>
-      <c r="D66" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E66" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" ht="119" x14ac:dyDescent="0.2">
-      <c r="A67" s="2">
-        <v>46229</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C67" s="4" t="s">
+    </row>
+    <row r="74" spans="1:8" ht="221" x14ac:dyDescent="0.2">
+      <c r="A74" s="2">
+        <v>46232</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C74" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="D67" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H67" s="3" t="s">
+      <c r="D74" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G74" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H74" s="3" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A68" s="2">
-        <v>46230</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E68" s="3" t="s">
+    <row r="75" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A75" s="2">
+        <v>46233</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="E75" s="4" t="s">
         <v>259</v>
       </c>
-      <c r="F68" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="G68" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H68" s="4" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" ht="255" x14ac:dyDescent="0.2">
-      <c r="A69" s="2">
-        <v>46232</v>
-      </c>
-      <c r="B69" s="4" t="s">
+      <c r="F75" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A76" s="2">
+        <v>46234</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="D76" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="C69" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="D69" s="3" t="s">
+      <c r="E76" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="F76" s="4" t="s">
         <v>263</v>
       </c>
-      <c r="E69" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H69" s="3" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A70" s="2">
-        <v>46233</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C70" s="4" t="s">
+      <c r="G76" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H76" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="D70" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="E70" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="F70" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H70" s="3" t="s">
+    </row>
+    <row r="77" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A77" s="2">
+        <v>46235</v>
+      </c>
+      <c r="B77" s="4" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A71" s="2">
-        <v>46234</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C71" s="4" t="s">
+      <c r="C77" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G77" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A78" s="2">
+        <v>46236</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G78" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H78" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="D71" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>270</v>
-      </c>
-      <c r="F71" s="4" t="s">
-        <v>269</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H71" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A72" s="2">
-        <v>46235</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>274</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E72" s="4" t="s">
+    </row>
+    <row r="79" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A79" s="2">
+        <v>46237</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C79" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="F72" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G72" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H72" s="4" t="s">
+      <c r="D79" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E79" s="4" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A73" s="2">
-        <v>46236</v>
-      </c>
-      <c r="B73" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C73" s="4" t="s">
+      <c r="F79" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="G79" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A80" s="2">
+        <v>46238</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="E80" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="D73" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="E73" s="4" t="s">
-        <v>280</v>
-      </c>
-      <c r="F73" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H73" s="3" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A74" s="2">
-        <v>46237</v>
-      </c>
-      <c r="B74" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C74" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E74" s="4" t="s">
+      <c r="F80" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G80" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H80" s="4" t="s">
         <v>282</v>
       </c>
-      <c r="F74" s="4" t="s">
+    </row>
+    <row r="81" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A81" s="2">
+        <v>46239</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="F81" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G81" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H81" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="G74" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H74" s="4" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" ht="85" x14ac:dyDescent="0.2">
-      <c r="A75" s="2">
-        <v>46238</v>
-      </c>
-      <c r="B75" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C75" s="4" t="s">
+    </row>
+    <row r="82" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A82" s="2">
+        <v>46240</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C82" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="D82" s="3" t="s">
         <v>287</v>
       </c>
-      <c r="D75" s="3" t="s">
+      <c r="E82" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="G82" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H82" s="3" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A83" s="2">
+        <v>46242</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C83" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="E75" s="4" t="s">
-        <v>284</v>
-      </c>
-      <c r="F75" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G75" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H75" s="4" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A76" s="2">
-        <v>46239</v>
-      </c>
-      <c r="B76" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D76" s="4" t="s">
-        <v>290</v>
-      </c>
-      <c r="E76" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="F76" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G76" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H76" s="4" t="s">
+      <c r="D83" s="3" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A77" s="2">
-        <v>46240</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C77" s="3" t="s">
+      <c r="E83" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="D77" s="3" t="s">
+      <c r="F83" s="4" t="s">
         <v>293</v>
       </c>
-      <c r="E77" s="3" t="s">
+      <c r="G83" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H83" s="4" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A84" s="2">
+        <v>46243</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="C84" s="4" t="s">
         <v>296</v>
       </c>
-      <c r="F77" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="G77" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H77" s="3" t="s">
+      <c r="D84" s="3" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A78" s="2">
-        <v>46242</v>
-      </c>
-      <c r="B78" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D78" s="3" t="s">
+      <c r="E84" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F84" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G84" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H84" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="E78" s="3" t="s">
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A85" s="2">
+        <v>46244</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C85" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="F85" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G85" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H85" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A86" s="2">
+        <v>46245</v>
+      </c>
+      <c r="B86" s="4" t="s">
         <v>298</v>
       </c>
-      <c r="F78" s="4" t="s">
+      <c r="C86" s="3" t="s">
         <v>299</v>
       </c>
-      <c r="G78" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H78" s="4" t="s">
+      <c r="E86" s="4" t="s">
+        <v>301</v>
+      </c>
+      <c r="F86" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H86" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A87" s="2">
+        <v>46247</v>
+      </c>
+      <c r="B87" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C87" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E87" s="3" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" ht="34" x14ac:dyDescent="0.2">
-      <c r="A79" s="2">
-        <v>46243</v>
-      </c>
-      <c r="B79" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C79" s="4" t="s">
+      <c r="F87" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G87" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H87" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A88" s="2">
+        <v>46248</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="C88" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E88" s="4" t="s">
         <v>302</v>
       </c>
-      <c r="D79" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="F79" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G79" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H79" s="3" t="s">
-        <v>303</v>
+      <c r="F88" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G88" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H88" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="D45:D48"/>
-    <mergeCell ref="G45:G48"/>
-    <mergeCell ref="H44:H48"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="H33:H34"/>
-    <mergeCell ref="E33:E34"/>
-    <mergeCell ref="F33:F34"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="B25:B30"/>
-    <mergeCell ref="H25:H28"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H30:H32"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D17:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F17:F20"/>
+    <mergeCell ref="G17:G20"/>
     <mergeCell ref="B17:B18"/>
     <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H16:H18"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="C20:C23"/>
-    <mergeCell ref="D20:D23"/>
-    <mergeCell ref="F20:F23"/>
-    <mergeCell ref="G20:G23"/>
-    <mergeCell ref="H12:H13"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D12:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F12:F15"/>
-    <mergeCell ref="G12:G15"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="H25:H28"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="D25:D28"/>
+    <mergeCell ref="F25:F28"/>
+    <mergeCell ref="G25:G28"/>
+    <mergeCell ref="B30:B35"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="B36:B40"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="G36:G37"/>
+    <mergeCell ref="H35:H37"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="G50:G53"/>
+    <mergeCell ref="H49:H53"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="G38:G39"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>